<commit_message>
Update answers workbook with Esportes filtered data
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iFLn21AiUGfBb2WhkxcsV
</commit_message>
<xml_diff>
--- a/analise/Respostas_por_bandeira_set26.xlsx
+++ b/analise/Respostas_por_bandeira_set26.xlsx
@@ -700,25 +700,25 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>128067</v>
+        <v>129419</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>111612</v>
+        <v>112757</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>-0.1284874323596242</v>
+        <v>-0.1287446201871441</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.006972912616052535</v>
+        <v>0.007008244539055316</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.007122890011826685</v>
+        <v>0.007103771827913123</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>385.624255256439</v>
+        <v>386.6242888092613</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>400.3964528805031</v>
+        <v>400.0502497440699</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>383239</v>
@@ -742,16 +742,16 @@
         <v>-49893.77000000002</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-49241.39509007004</v>
+        <v>-49339.95949590092</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>7183.811663418308</v>
+        <v>4551.278128756475</v>
       </c>
       <c r="R5" s="5" t="n">
-        <v>13069.71551342921</v>
+        <v>11753.06592954387</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>-20905.90208677753</v>
+        <v>-16858.1545623995</v>
       </c>
     </row>
     <row r="6">
@@ -1020,19 +1020,19 @@
         <v>465538</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>501727</v>
+        <v>502872</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>0.013</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.009116238702392754</v>
+        <v>0.009107413209396047</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>300</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>353.3317613460429</v>
+        <v>353.3328704265586</v>
       </c>
       <c r="H3" s="5" t="n">
         <v>1646605.94</v>
@@ -1041,13 +1041,13 @@
         <v>1237130.99</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>141137.1</v>
+        <v>145602.6</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-584576.3713693771</v>
+        <v>-587241.8713693772</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>243932.1750352344</v>
+        <v>244257.2450402343</v>
       </c>
     </row>
     <row r="4">
@@ -4774,40 +4774,40 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>21730</v>
+        <v>23082</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>19476</v>
+        <v>20621</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-0.1037275655775426</v>
+        <v>-0.1066198769604021</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.008513575701794753</v>
+        <v>0.008621436617277533</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.007496405832819881</v>
+        <v>0.007371126521507202</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>391.3178378810812</v>
+        <v>395.4752261859297</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>438.0347260890411</v>
+        <v>434.7246053289474</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>72393.80000800002</v>
+        <v>78699.570011</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>63953.070009</v>
+        <v>66078.14001</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-7509.232637737324</v>
+        <v>-8390.938471409369</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>-7752.163039624837</v>
+        <v>-10196.39715932933</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>6820.665678362149</v>
+        <v>5965.905629738696</v>
       </c>
     </row>
     <row r="4">
@@ -4832,25 +4832,25 @@
         <v>0.007065175976224431</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>384.1365253333333</v>
+        <v>384.1365253375706</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>391.9292912650231</v>
+        <v>391.9292912711864</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>271968.659936</v>
+        <v>271968.659939</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>254362.110031</v>
+        <v>254362.110035</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-36315.50582515697</v>
+        <v>-36315.50582555755</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>13651.4508304903</v>
+        <v>13651.45083064088</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>5057.505089666653</v>
+        <v>5057.50509091668</v>
       </c>
     </row>
     <row r="5">
@@ -5003,16 +5003,16 @@
         <v>159115.529996</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>137053.130018</v>
+        <v>137053.130021</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>-22062.39997799997</v>
+        <v>-22062.39997499998</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>google / organic</t>
+          <t>(direct) / (none)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5021,40 +5021,40 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>4795</v>
+        <v>861</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4353</v>
+        <v>925</v>
       </c>
       <c r="E11" t="n">
-        <v>-9.217935349322214</v>
+        <v>7.433217189314756</v>
       </c>
       <c r="F11" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G11" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4796663190823775</v>
+        <v>1.509872241579559</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2756719503790489</v>
+        <v>0.6486486486486486</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>8691.350006000001</v>
+        <v>6065.790005</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>4903.449998</v>
+        <v>2125.070002</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>-3787.900008000001</v>
+        <v>-3940.720002999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>google / cpc</t>
+          <t>google / organic</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5063,118 +5063,118 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>12577</v>
+        <v>4795</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>11292</v>
+        <v>4353</v>
       </c>
       <c r="E12" t="n">
-        <v>-10.2170628925817</v>
+        <v>-9.217935349322214</v>
       </c>
       <c r="F12" t="n">
-        <v>136</v>
+        <v>23</v>
       </c>
       <c r="G12" t="n">
-        <v>112</v>
+        <v>12</v>
       </c>
       <c r="H12" t="n">
-        <v>1.081338952055339</v>
+        <v>0.4796663190823775</v>
       </c>
       <c r="I12" t="n">
-        <v>0.991852639036486</v>
+        <v>0.2756719503790489</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>51921.52000200001</v>
+        <v>8691.350006000001</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>49035.140008</v>
+        <v>4903.449998</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>-2886.37999400001</v>
+        <v>-3787.900008000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>linktr.ee / referral</t>
+          <t>google / cpc</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>622</v>
+        <v>12577</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>464</v>
+        <v>11292</v>
       </c>
       <c r="E13" t="n">
-        <v>-25.40192926045016</v>
+        <v>-10.2170628925817</v>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>136</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>112</v>
       </c>
       <c r="H13" t="n">
-        <v>0.964630225080386</v>
+        <v>1.081338952055339</v>
       </c>
       <c r="I13" t="n">
-        <v>0.646551724137931</v>
+        <v>0.991852639036486</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>3666.159998</v>
+        <v>51921.520001</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>798.3099980000001</v>
+        <v>49035.140007</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>-2867.849999999999</v>
+        <v>-2886.379993999995</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lojaspaqueta.com.br / referral</t>
+          <t>linktr.ee / referral</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>787</v>
+        <v>622</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>681</v>
+        <v>464</v>
       </c>
       <c r="E14" t="n">
-        <v>-13.46886912325286</v>
+        <v>-25.40192926045016</v>
       </c>
       <c r="F14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H14" t="n">
-        <v>1.143583227445997</v>
+        <v>0.964630225080386</v>
       </c>
       <c r="I14" t="n">
-        <v>1.3215859030837</v>
+        <v>0.646551724137931</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>5426.140004000001</v>
+        <v>3666.159998</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>3615.310005</v>
+        <v>798.3099980000001</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>-1810.829999</v>
+        <v>-2867.85</v>
       </c>
     </row>
     <row r="15">
@@ -5185,44 +5185,44 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1704</v>
+        <v>787</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1421</v>
+        <v>681</v>
       </c>
       <c r="E15" t="n">
-        <v>-16.60798122065728</v>
+        <v>-13.46886912325286</v>
       </c>
       <c r="F15" t="n">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="G15" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="H15" t="n">
-        <v>2.758215962441315</v>
+        <v>1.143583227445997</v>
       </c>
       <c r="I15" t="n">
-        <v>2.814919071076706</v>
+        <v>1.3215859030837</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>17613.239974</v>
+        <v>5426.140004000001</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>15912.570009</v>
+        <v>3615.310004999999</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>-1700.669964999997</v>
+        <v>-1810.829999000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(direct) / (none)</t>
+          <t>lojaspaqueta.com.br / referral</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -5231,97 +5231,97 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>4698</v>
+        <v>1704</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7294</v>
+        <v>1421</v>
       </c>
       <c r="E16" t="n">
-        <v>55.25755640698169</v>
+        <v>-16.60798122065728</v>
       </c>
       <c r="F16" t="n">
-        <v>69</v>
+        <v>47</v>
       </c>
       <c r="G16" t="n">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="H16" t="n">
-        <v>1.468710089399744</v>
+        <v>2.758215962441315</v>
       </c>
       <c r="I16" t="n">
-        <v>0.945982999725802</v>
+        <v>2.814919071076706</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>29457.629993</v>
+        <v>17613.239974</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>27991.800015</v>
+        <v>15912.570009</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>-1465.829978000002</v>
+        <v>-1700.669964999999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>l.instagram.com / referral</t>
+          <t>(direct) / (none)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>34</v>
+        <v>4698</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>9</v>
+        <v>7294</v>
       </c>
       <c r="E17" t="n">
-        <v>-73.52941176470588</v>
+        <v>55.25755640698169</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="H17" t="n">
-        <v>5.88235294117647</v>
+        <v>1.468710089399744</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>0.945982999725802</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>1178.950004</v>
+        <v>29457.629995</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>0</v>
+        <v>27991.800016</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>-1178.950004</v>
+        <v>-1465.829979000002</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bing / organic</t>
+          <t>l.instagram.com / referral</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E18" t="n">
-        <v>-42.30769230769231</v>
+        <v>-73.52941176470588</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
@@ -5330,25 +5330,25 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>7.692307692307693</v>
+        <v>5.88235294117647</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>849.979997</v>
+        <v>1178.950003</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>-849.979997</v>
+        <v>-1178.950003</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cloud.email.portaldocartao.com.br / referral</t>
+          <t>bing / organic</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5357,40 +5357,40 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>121</v>
+        <v>26</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E19" t="n">
-        <v>-71.07438016528927</v>
+        <v>-42.30769230769231</v>
       </c>
       <c r="F19" t="n">
         <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>1.652892561983471</v>
+        <v>7.692307692307693</v>
       </c>
       <c r="I19" t="n">
-        <v>2.857142857142857</v>
+        <v>0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>779.979998</v>
+        <v>849.979997</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>134.990002</v>
+        <v>0</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>-644.989996</v>
+        <v>-849.979997</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>crm / web_push</t>
+          <t>cloud.email.portaldocartao.com.br / referral</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5399,40 +5399,40 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2420</v>
+        <v>121</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1607</v>
+        <v>35</v>
       </c>
       <c r="E20" t="n">
-        <v>-33.59504132231405</v>
+        <v>-71.07438016528927</v>
       </c>
       <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
       <c r="H20" t="n">
-        <v>0.04132231404958678</v>
+        <v>1.652892561983471</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>2.857142857142857</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>598.49</v>
+        <v>779.979998</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>0</v>
+        <v>134.990002</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>-598.49</v>
+        <v>-644.989996</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>m.facebook.com / referral</t>
+          <t>crm / web_push</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5441,34 +5441,34 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>440</v>
+        <v>2420</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>171</v>
+        <v>1607</v>
       </c>
       <c r="E21" t="n">
-        <v>-61.13636363636363</v>
+        <v>-33.59504132231405</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.04132231404958678</v>
       </c>
       <c r="I21" t="n">
-        <v>0.5847953216374269</v>
+        <v>0</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>549.960003</v>
+        <v>598.49</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>309.970002</v>
+        <v>0</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>-239.990001</v>
+        <v>-598.49</v>
       </c>
     </row>
     <row r="22">
@@ -5588,7 +5588,7 @@
         <v>4565.209999</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>994.909999</v>
+        <v>994.9099989999995</v>
       </c>
     </row>
     <row r="25">
@@ -5669,10 +5669,10 @@
         <v>0</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>6081.850005</v>
+        <v>6081.850004999999</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>6081.850005</v>
+        <v>6081.850004999999</v>
       </c>
     </row>
     <row r="27"/>
@@ -5728,16 +5728,16 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.2165375854214123</v>
+        <v>0.7309945015539087</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.2658062665806267</v>
+        <v>0.7209362978418205</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>4.926868115921438</v>
+        <v>-1.005820371208821</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0.2275294659046403</v>
+        <v>-0.01375961609930998</v>
       </c>
     </row>
     <row r="32">
@@ -5752,16 +5752,16 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0.04951258854057087</v>
+        <v>0.05772218134249039</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>0.1254315925766077</v>
+        <v>0.06376051370172742</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>7.591900403603683</v>
+        <v>0.6038332359237022</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>1.533327306727831</v>
+        <v>0.1046102593283682</v>
       </c>
     </row>
     <row r="33">
@@ -5779,13 +5779,13 @@
         <v>0.7917847025495751</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>0.92</v>
+        <v>0.7475177304964539</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>12.82152974504249</v>
+        <v>-4.426697205312125</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0.1619320214669051</v>
+        <v>-0.0559078394803284</v>
       </c>
     </row>
     <row r="34">
@@ -5803,13 +5803,13 @@
         <v>0.4633273703041145</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0.09069658719027583</v>
+        <v>0.3681214421252372</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>-37.26307831138386</v>
+        <v>-9.52059281788773</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>-0.8042494508132657</v>
+        <v>-0.2054830650656078</v>
       </c>
     </row>
     <row r="35">
@@ -5851,13 +5851,13 @@
         <v>0.3559928443649374</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>0.06778868630201028</v>
+        <v>0.2751423149905123</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>-28.82041580629271</v>
+        <v>-8.085052937442505</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>-0.8095785143576696</v>
+        <v>-0.2271127935693649</v>
       </c>
     </row>
     <row r="37">
@@ -5872,16 +5872,16 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>0.01395609790307876</v>
+        <v>0.01627013326792576</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>0.007822615451014243</v>
+        <v>0.01311386452021344</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>-0.6133482452064514</v>
+        <v>-0.3156268747712325</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>-0.4394840516783312</v>
+        <v>-0.1939915731320072</v>
       </c>
     </row>
     <row r="38">
@@ -5896,16 +5896,16 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>0.7719343531777301</v>
+        <v>0.7711639495206629</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>0.7275880428995208</v>
+        <v>0.7316562805474096</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>-4.434631027820924</v>
+        <v>-3.950766897325331</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>-0.05744829219693881</v>
+        <v>-0.05123121872827474</v>
       </c>
     </row>
     <row r="39">
@@ -5920,16 +5920,16 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>0.06386948027948397</v>
+        <v>0.06372032588846747</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>0.07219620306096847</v>
+        <v>0.07208316806880571</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.8326722781484497</v>
+        <v>0.8362842180338239</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.1303709180824379</v>
+        <v>0.1312429285904171</v>
       </c>
     </row>
     <row r="40">
@@ -6040,16 +6040,16 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>0.0120206269029726</v>
+        <v>0.01199255513414805</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>0.01290039307518608</v>
+        <v>0.01288019539486045</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>0.08797661722134853</v>
+        <v>0.08876402607123929</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.07318804412737623</v>
+        <v>0.07401594162238978</v>
       </c>
     </row>
     <row r="45">
@@ -6230,19 +6230,19 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>16921</v>
+        <v>17617</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>0.006028012528810354</v>
+        <v>0.006527785661576886</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>445.9423530784314</v>
+        <v>441.3642609826086</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>45486.120014</v>
+        <v>50756.890013</v>
       </c>
     </row>
     <row r="57">
@@ -6257,19 +6257,19 @@
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>2766</v>
+        <v>3299</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.005061460592913955</v>
+        <v>0.007578053955744165</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>491.8528573571429</v>
+        <v>461.88919984</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>6885.940003</v>
+        <v>11547.229996</v>
       </c>
     </row>
     <row r="58">
@@ -6284,19 +6284,19 @@
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>14099</v>
+        <v>14262</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>0.006241577416838073</v>
+        <v>0.006310475389145982</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>438.6384092159091</v>
+        <v>435.6628890777777</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>38600.180011</v>
+        <v>39209.66001699999</v>
       </c>
     </row>
     <row r="59">
@@ -6336,19 +6336,19 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>18642</v>
+        <v>18772</v>
       </c>
       <c r="D60" s="3" t="n">
         <v>130</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>0.00697350069735007</v>
+        <v>0.006925207756232687</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>411.5460001230769</v>
+        <v>411.5460001461539</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>53500.980016</v>
+        <v>53500.98001900001</v>
       </c>
     </row>
     <row r="61">
@@ -6363,13 +6363,13 @@
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>2691</v>
+        <v>2821</v>
       </c>
       <c r="D61" s="3" t="n">
         <v>17</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0.0063173541434411</v>
+        <v>0.006026231832683446</v>
       </c>
       <c r="F61" s="5" t="n">
         <v>527.0723531176471</v>
@@ -6399,10 +6399,10 @@
         <v>0.007102897730844176</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>394.1659293185841</v>
+        <v>394.1659293451328</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>44540.750013</v>
+        <v>44540.75001600001</v>
       </c>
     </row>
     <row r="63">
@@ -6442,19 +6442,19 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>19528</v>
+        <v>19833</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>106</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>0.005428103236378533</v>
+        <v>0.005344627640800685</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>423.3349059622641</v>
+        <v>423.3349059622643</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>44873.500032</v>
+        <v>44873.50003200001</v>
       </c>
     </row>
     <row r="65">
@@ -6469,13 +6469,13 @@
         </is>
       </c>
       <c r="C65" s="3" t="n">
-        <v>3061</v>
+        <v>3366</v>
       </c>
       <c r="D65" s="3" t="n">
         <v>25</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.008167265599477294</v>
+        <v>0.00742721330956625</v>
       </c>
       <c r="F65" s="5" t="n">
         <v>498.14279984</v>
@@ -6505,10 +6505,10 @@
         <v>0.004930306165926106</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>400.2460498271604</v>
+        <v>400.2460498271607</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>32419.930036</v>
+        <v>32419.93003600001</v>
       </c>
     </row>
     <row r="67">

</xml_diff>

<commit_message>
Add quick-answers, group origins, monthly history and October vs target sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iFLn21AiUGfBb2WhkxcsV
</commit_message>
<xml_diff>
--- a/analise/Respostas_por_bandeira_set26.xlsx
+++ b/analise/Respostas_por_bandeira_set26.xlsx
@@ -7,13 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupo e Diadora" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oscar web" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oscar app" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paq Esportes web" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paq Calçados web" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diadora web" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perguntas rápidas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grupo e Diadora" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oscar web" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oscar app" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paq Esportes web" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paq Calçados web" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diadora web" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origens Grupo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico mensal" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outubro vs meta" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -69,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -78,6 +82,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,6 +450,1170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Respostas rápidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Pergunta</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Resposta</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Onde está</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Qual bandeira teve o maior gap vs meta em setembro?</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes: -R$ 215.523 (60,7% da meta). Depois Oscar web -R$ 115.831 (81,4%), Diadora -R$ 72.514 (72,7%), App -R$ 59.952 (81,8%), Calçados -R$ 18.169 (87,6%). Grupo -R$ 409.475 (75,1%).</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Resumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Qual origem/mídia teve o maior gap?</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Não existe meta por origem. Pela contribuição à piora de setembro sobre agosto (receita captada GA4), o google / cpc: -R$ 251 mil no Grupo (Oscar web -R$ 200 mil, App -R$ 29 mil, Esportes -R$ 25 mil, Calçados +R$ 3 mil). Por origem x device: google / cpc mobile -R$ 148 mil, google / cpc desktop -R$ 73 mil, google / cpc iOS (app) -R$ 24 mil. Diadora: Meta Ads -R$ 12 mil.</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Origens Grupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Qual foi a CVR de Paquetá Calçados em setembro?</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>0,64% (450 transações / 69.961 sessões, GA4), igual a agosto (0,64%). Pela planilha de captado (771 pedidos) seria cerca de 1,1%.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Resumo, aba Paq Calçados web</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>CVR de setembro por bandeira</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Oscar web 1,01%; App 1,13% (01-24/09); Esportes 0,71%; Calçados 0,64%; Diadora 1,53%; Grupo 0,91% (meta 1,30%).</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Resumo, Grupo e Diadora</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Variação de sessões Set vs Ago</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Oscar web -6,4%; App -8,8%; Esportes -12,9%; Calçados -0,4%; Diadora +8,5%; Grupo -7,2%.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Resumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>O gap foi volume, conversão ou ticket?</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Oscar web: conversão. App: conversão e volume. Esportes: volume (e meta 43% acima de agosto). Calçados: ticket. Diadora: meta 47% acima de agosto; contra as metas de KPI, volume (43%), conversão (29%) e ticket (28%). Grupo: conversão.</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Resumo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Qual bandeira tem o maior gap de outubro (01-05) vs meta?</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Diadora: -R$ 22.892 (43,8% da meta). Em R$, entre as bandeiras do Grupo: Oscar web -R$ 21.391 (75,3%), App -R$ 17.069 (67,0%), Esportes -R$ 4.848 (91,4%); Calçados +R$ 6.388 (129,5%). Grupo (4 bandeiras) -R$ 36.841 (83,0%). Faturado ainda amadurece.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Outubro vs meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Onde está a perda no funil?</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Ver abas por bandeira (taxa de passagem por device, Ago vs Set) e o resumo do chat.</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>abas por bandeira</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Histórico mensal</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>CVR e sessões de mai a out por bandeira.</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Histórico mensal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Histórico mensal (mai a out/26; out = 01 a 05; Diadora: até jul as sessões estão infladas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bandeira</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>AnoMes</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sessões</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CVR</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>TKM</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Receita GA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>202605</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>318371</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.009611428176561307</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>344.4644727720828</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>1054061.286682573</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>202606</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>303083</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.01072973409924014</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>360.1643693967197</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1171254.529278133</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>202607</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>343990</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.01287246722288439</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>394.1893495229506</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1745470.439687625</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>202608</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>280282</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.01132430908870352</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>332.0564378973676</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1053947.133886245</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>202609</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>247080</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0.009713453132588635</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>352.7904436360002</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>846697.0647264005</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>202610</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>32037</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.01030058994287855</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>367.634362366622</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>121319.3395809853</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>202605</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>176562</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.006569930109536593</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>444.7366473426439</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>515894.510917467</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>202606</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>265501</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.005551768166598242</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>477.4259376818879</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>703725.8321431028</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>202607</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>191392</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0.004817338237752884</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>441.7304615489375</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>407275.4855481203</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>202608</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>131645</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.006213680732272399</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>409.4396360919952</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>334921.622323252</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>202609</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>112874</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.005971259989014299</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>451.5438877765191</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>304340.5803613739</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>202610</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>17500</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.006571428571428572</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>476.6549229117765</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>54815.31613485429</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>202605</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>113040</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0.006033262561924982</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>297.5301026495601</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>202915.530007</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>202606</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>97133</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.006228573193456395</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>285.3284462181819</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>172623.709962</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>202607</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>83946</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0.007326138231720391</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>291.8709593235773</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>179500.639984</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>202608</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>71643</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0.006518431668132267</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>286.80931475803</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>133939.949992</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>202609</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>69700</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0.006456241032998565</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>266.8136001333334</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>120066.12006</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>202610</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>11879</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0.007828941830120381</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>263.9444089354839</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>24546.830031</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>202605</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>127207</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0.005903763157687863</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>230.540466011984</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>173135.889975</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>202606</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>80600</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.006538461538461538</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>265.7214041574953</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>140035.179991</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>202607</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>97469</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0.005458145666827402</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>252.5614473984963</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>134362.690016</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>202608</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>56074</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0.01551521204123123</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>171.4177930862069</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>149133.479985</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>202609</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>58033</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>0.01550841762445505</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>188.4096666844445</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>169568.700016</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>202610</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>13833</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>0.006072435480373021</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>169.6426188452381</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>14249.979983</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app) (CVR = sessões com compra / sessões)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>202605</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>104690</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0.009838571019199542</v>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app) (CVR = sessões com compra / sessões)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>202606</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>84068</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0.01271589665508874</v>
+      </c>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app) (CVR = sessões com compra / sessões)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>202607</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>89821</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>0.01433963104396522</v>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app) (CVR = sessões com compra / sessões)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>202608</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>80537</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0.01193240373989595</v>
+      </c>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app) (CVR = sessões com compra / sessões)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>202609</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>68215</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>0.0110239683354101</v>
+      </c>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app) (CVR = sessões com compra / sessões)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>202610</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>10846</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>0.008297990042411949</v>
+      </c>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Outubro 01-05: faturado vs meta proporcional por dia (planilha de metas, posição de 06/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Bandeira</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Meta 01-05/10</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Faturado 01-05/10</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Atingimento</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Oscar web</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>86538</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>65147</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>0.7528137927846726</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>-21391</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Oscar app</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>51760</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>34692</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0.6702472952086553</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>-17068</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>56412</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>51564</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0.9140608381195491</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>-4848</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>21634</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>28023</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1.295322178053065</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>6389</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GRUPO (4 bandeiras)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>216344</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>179426</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0.829355101135229</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>-36918</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Diadora (site)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>40765</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>17873</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0.4384398380964062</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>-22892</v>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Diadora: gap de outubro (01-05) vs metas de KPI de outubro</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Alavanca (Diadora)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Meta pro-rata</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Real (GA4)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Efeito no gap (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sessões</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>20322.58064516129</v>
+      </c>
+      <c r="C13" t="n">
+        <v>13816</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>-7764.675575042232</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CVR</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.0125</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.006079907353792704</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>-14501.76074841333</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TKM</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>175</v>
+      </c>
+      <c r="C15" t="n">
+        <v>169.6428571428571</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>-625.5636765444378</v>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Faturado de 01 a 05/10 ainda amadurece (aprovação e faturamento): na Oscar web o faturado é 44% do captado do GA4, contra 57% em setembro. O gap de outubro tende a estar superestimado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Outubro 04/10 (domingo) tem faturado muito baixo em todas as bandeiras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Metas de KPI de outubro só existem para o Grupo e a Diadora (Diadora: 126 mil sessões, CVR 1,25%, TKM R$ 175).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -876,8 +2047,6 @@
         <v>-19242.09085229585</v>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -918,7 +2087,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1090,9 +2259,6 @@
         <v>-28431.29998199997</v>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -1105,7 +2271,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1332,8 +2498,6 @@
         <v>289.5466633333333</v>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -2111,8 +3275,6 @@
         <v>17757.63999100001</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
@@ -2656,8 +3818,6 @@
         <v>-0.6453537936913896</v>
       </c>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -3029,7 +4189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3213,8 +4373,6 @@
         <v>-6828.31892075865</v>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -3998,8 +5156,6 @@
         <v>20763.89999200001</v>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
@@ -4375,8 +5531,6 @@
         <v>-0.07582643054475291</v>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
@@ -4669,7 +5823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4887,7 +6041,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L5" s="5" t="n">
         <v>0</v>
@@ -4896,8 +6050,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -5675,8 +6827,6 @@
         <v>6081.850004999999</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
@@ -6172,8 +7322,6 @@
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="4" t="n"/>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -6541,7 +7689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6768,8 +7916,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -7553,8 +8699,6 @@
         <v>2796.110037999992</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
@@ -8050,8 +9194,6 @@
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="4" t="n"/>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -8419,7 +9561,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8637,7 +9779,7 @@
         <v>178.620002</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L5" s="5" t="n">
         <v>0</v>
@@ -8646,8 +9788,6 @@
         <v>178.620002</v>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
@@ -9428,8 +10568,6 @@
         <v>14502.51001100001</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
@@ -9937,8 +11075,6 @@
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="4" t="n"/>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
@@ -10301,6 +11437,1445 @@
       </c>
       <c r="G67" s="5" t="n">
         <v>178.620002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GRUPO (Oscar web + App + Esportes + Calçados): origem, variação de receita captada Set vs Ago (R$ GA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Sessoes_A</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sessoes_S</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CVR_A</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>CVR_S</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Receita_A</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Receita_S</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>dRec</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>240919</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>223777</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.0105346610271502</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0.008280565026790063</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>887331.6599719999</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>636151.100001</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>-251180.5599709999</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Meta Ads (soma das grafias)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>52186</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>33239</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0.003717472118959108</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.00394115346430398</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>61443.42997300001</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>48730.870019</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>-12712.559954</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>firebase / app_push</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1034</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>237</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.03094777562862669</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0.04219409282700422</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>14680.45001</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>3125.649998</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>-11554.800012</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ntp.msn.com / referral</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>315</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>149</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.1677852348993289</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>16639.340002</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>8080.720001</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>-8558.620000999998</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>awin / referral</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>968</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>551</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0.03615702479338843</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0.02540834845735027</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>12852.009981</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>5027.379999000001</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>-7824.629982</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>google-play / organic</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>3694</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>3085</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0.01434759068760152</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.008752025931928687</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>16757.609994</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>10579.339994</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>-6178.27</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bonifiq / email</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1546</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>231</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0.0129366106080207</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0.02164502164502164</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>7372.100007</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1299.320003</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>-6072.780004</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>awin / (not set)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>1276</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>429</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0.01959247648902821</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.02564102564102564</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>9371.580008999999</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>3676.779999</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>-5694.800010000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ig / source</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>8085</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>7803</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0.005318491032776747</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0.004998077662437524</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>16675.020013</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>11529.589994</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>-5145.430019000003</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>(data not available)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2239</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>2478</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.01786511835640911</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.01089588377723971</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>12852.929999</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>8244.420017</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>-4608.509982</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>lojaspaqueta.com.br / referral</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2510</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>2113</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.02231075697211156</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.02318977756743966</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>23039.379978</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>19527.880014</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>-3511.499964000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>referral / gaston</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>1569</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>948</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.008922880815806247</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.006329113924050633</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>4605.100006000001</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>1436.650001</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>-3168.450005</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>linktr.ee / referral</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2652</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>2256</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>0.004147812971342383</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>0.005319148936170213</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>5521.23</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>3365.589994</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>-2155.640006</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>bing / organic</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>1803</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1635</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0.02551303383250139</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0.01529051987767584</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>13996.22997</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>12039.320007</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>-1956.909962999997</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pelando.com.br / referral</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>657</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0.0060882800608828</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>1379.879996</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>-1379.879996</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>84537</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>84217</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0.01807492577214711</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0.01765676763598798</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>520907.4199640001</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>528516.0501550001</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>7608.630190999966</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>crm / web_push</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>10162</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>9014</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>0.007380436921865774</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0.0110938540048813</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>29088.47998599999</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>39788.29002499999</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>10699.810039</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>crm / app_push</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>8699</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>8692</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0.005977698586044373</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.01046939714680166</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>17571.93999</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>30459.59998</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>12887.65998999999</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>(not set)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>15824</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>17457</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0.009036905965621841</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0.01042561723091024</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>45234.049987</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>61329.45001100001</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>16095.40002400001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>google / organic</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>77583</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>80026</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.005387778250389905</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.005673156224227126</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>128083.85002</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>159039.490009</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>30955.63998900001</v>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>GRUPO: origem x device, maiores perdas</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Sessoes_A</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Sessoes_S</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>CVR_A</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>CVR_S</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Receita_A</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Receita_S</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>dRec</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>170248</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>161621</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0.008099948310699686</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>0.005970758750409909</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>464426.4899459999</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>316076.920068</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>-148349.5698779999</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>39852</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>32324</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.01927130382414935</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.0175102091325331</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>285919.07999</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>212867.689981</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>-73051.39000899998</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>4477</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>3150</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>0.02255974983247711</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>0.01873015873015873</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>47093.700008</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>22981.559986</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>-24112.140022</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Meta Ads (soma das grafias)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>49492</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>31274</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.00365715671219591</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.003901004028905801</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>57095.16997800001</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>45082.330021</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>-12012.839957</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ntp.msn.com / referral</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>314</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>149</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0.1337579617834395</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>0.1677852348993289</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>16639.340002</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>8080.720001</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>-8558.620000999998</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>firebase / app_push</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>404</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.04455445544554455</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.06542056074766354</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>9449.380004999999</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>2119.899997</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>-7329.480007999999</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>google-play / organic</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>3681</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>3085</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.01439826134202662</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>0.008752025931928687</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>16757.609994</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>10579.339994</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>-6178.27</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ig / source</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>7573</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>7321</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.005149874554337779</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.004644174293129354</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>15340.600008</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>10069.72</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>-5270.880008000003</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>(not set)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>11758</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>13807</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.006378635822418779</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>0.003911059607445499</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>22913.259992</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>17656.220022</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>-5257.039969999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>25988</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>26096</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.01104355856549176</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.01007817290006131</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>89028.440023</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>84224.92996600001</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>-4803.510056999992</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>awin / referral</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>395</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>263</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.0430379746835443</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>0.01520912547528517</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>5736.079991000001</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>1063.779998</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>-4672.299993000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>awin / (not set)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>974</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>189</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0.01334702258726899</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0.01587301587301587</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>5602.800003</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>1245.960001</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>-4356.840002000001</v>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>DIADORA (à parte): origem</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Sessoes_A</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Sessoes_S</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>CVR_A</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>CVR_S</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Receita_A</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Receita_S</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>dRec</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Meta Ads (soma das grafias)</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>10341</v>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>5596</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>0.009186732424330336</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0.008220157255182273</v>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>20354.25</v>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>7995.240001000001</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>-12359.009999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>(data not available)</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>486</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>436</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>0.02880658436213992</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>0.02981651376146789</v>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>2335.070002</v>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>1547.240002</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>-787.8299999999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>bing / organic</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>0.03252032520325204</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>0.02857142857142857</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>804.419997</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>430.440002</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>-373.9799949999999</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Instagram / referral</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>178</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>233</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>0.01123595505617977</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>0.004291845493562232</v>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>410.969997</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>80.489998</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>-330.479999</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>l.wl.co / referral</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="C47" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>528.000002</v>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>252.490001</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>-275.510001</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>duckduckgo / organic</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C48" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>409.980001</v>
+      </c>
+      <c r="G48" s="5" t="n">
+        <v>182.400001</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>-227.58</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>edrone / email</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>0.02857142857142857</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="5" t="n">
+        <v>97.49000100000001</v>
+      </c>
+      <c r="G49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>-97.49000100000001</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>a45d8dfd3c74c42841f31013bfea46c5.safeframe.googlesyndication.com / referral</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="5" t="n">
+        <v>76.48999999999999</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>-76.48999999999999</v>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>Google CPC por bandeira (R$ GA, Set vs Ago)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Bandeira</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Google CPC dRec</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Diadora (web)</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>17443.00998900001</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app)</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>-28915.65007899999</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>-200378.9800009999</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web)</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>3062.850077999994</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web)</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>-24948.77996899997</v>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Não existe meta por origem. A coluna dRec é a contribuição da origem à piora de setembro sobre agosto; o gap vs meta = piora + meta acima de agosto (ver Resumo). App: a base de setembro inclui compra duplicada após 25/09.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix October group gap figure
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iFLn21AiUGfBb2WhkxcsV
</commit_message>
<xml_diff>
--- a/analise/Respostas_por_bandeira_set26.xlsx
+++ b/analise/Respostas_por_bandeira_set26.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Diadora: -R$ 22.892 (43,8% da meta). Em R$, entre as bandeiras do Grupo: Oscar web -R$ 21.391 (75,3%), App -R$ 17.069 (67,0%), Esportes -R$ 4.848 (91,4%); Calçados +R$ 6.388 (129,5%). Grupo (4 bandeiras) -R$ 36.841 (83,0%). Faturado ainda amadurece.</t>
+          <t>Diadora: -R$ 22.892 (43,8% da meta). Em R$, entre as bandeiras do Grupo: Oscar web -R$ 21.391 (75,3%), App -R$ 17.068 (67,0%), Esportes -R$ 4.848 (91,4%); Calçados +R$ 6.388 (129,5%). Grupo (4 bandeiras) -R$ 36.918 (83,0%). Faturado ainda amadurece.</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -1501,8 +1501,6 @@
         <v>-22892</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -1580,8 +1578,6 @@
         <v>-625.5636765444378</v>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -12073,8 +12069,6 @@
         <v>30955.63998900001</v>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
@@ -12525,8 +12519,6 @@
         <v>-4356.840002000001</v>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
@@ -12798,8 +12790,6 @@
         <v>-76.48999999999999</v>
       </c>
     </row>
-    <row r="51"/>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
@@ -12869,8 +12859,6 @@
         <v>-24948.77996899997</v>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Restore October 01-05 window; add October origin sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iFLn21AiUGfBb2WhkxcsV
</commit_message>
<xml_diff>
--- a/analise/Respostas_por_bandeira_set26.xlsx
+++ b/analise/Respostas_por_bandeira_set26.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outubro vs meta" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs completos" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funil completo" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outubro origem" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5105,7 +5106,6 @@
       <c r="J3" s="6" t="n">
         <v>0.58650132140679</v>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5144,7 +5144,6 @@
       <c r="J4" s="6" t="n">
         <v>0.1081455805892548</v>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5183,7 +5182,6 @@
       <c r="J5" s="6" t="n">
         <v>0.8044871794871795</v>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5265,7 +5263,6 @@
       <c r="J7" s="6" t="n">
         <v>0.8941798941798942</v>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5304,7 +5301,6 @@
       <c r="J8" s="6" t="n">
         <v>0.058578856152513</v>
       </c>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5343,7 +5339,6 @@
       <c r="J9" s="6" t="n">
         <v>0.08700173310225304</v>
       </c>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5382,7 +5377,6 @@
       <c r="J10" s="6" t="n">
         <v>0.7681249740329885</v>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5421,7 +5415,6 @@
       <c r="J11" s="6" t="n">
         <v>0.06328429251406317</v>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5460,7 +5453,6 @@
       <c r="J12" s="6" t="n">
         <v>0.6675213675213675</v>
       </c>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5499,7 +5491,6 @@
       <c r="J13" s="6" t="n">
         <v>0.3277848911651728</v>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5538,7 +5529,6 @@
       <c r="J14" s="6" t="n">
         <v>0.65234375</v>
       </c>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5577,7 +5567,6 @@
       <c r="J15" s="6" t="n">
         <v>0.009032886196451753</v>
       </c>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5616,7 +5605,6 @@
       <c r="J16" s="6" t="n">
         <v>0.04224361748160969</v>
       </c>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5655,7 +5643,6 @@
       <c r="J17" s="6" t="n">
         <v>0.3069461285293608</v>
       </c>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5694,7 +5681,6 @@
       <c r="J18" s="6" t="n">
         <v>0.3205417607223476</v>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5733,7 +5719,6 @@
       <c r="J19" s="6" t="n">
         <v>0.4753521126760563</v>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5772,7 +5757,6 @@
       <c r="J20" s="6" t="n">
         <v>0.4333333333333333</v>
       </c>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5811,7 +5795,6 @@
       <c r="J21" s="6" t="n">
         <v>0.6581196581196581</v>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5850,7 +5833,6 @@
       <c r="J22" s="6" t="n">
         <v>0.04345372460496614</v>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5889,7 +5871,6 @@
       <c r="J23" s="6" t="n">
         <v>0.1523702031602709</v>
       </c>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5928,7 +5909,6 @@
       <c r="J24" s="6" t="n">
         <v>0.5415807560137457</v>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5967,7 +5947,6 @@
       <c r="J25" s="6" t="n">
         <v>0.3565989847715736</v>
       </c>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6006,7 +5985,6 @@
       <c r="J26" s="6" t="n">
         <v>0.4946619217081851</v>
       </c>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6045,7 +6023,6 @@
       <c r="J27" s="6" t="n">
         <v>0.5827338129496403</v>
       </c>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6084,7 +6061,6 @@
       <c r="J28" s="6" t="n">
         <v>0.5308641975308642</v>
       </c>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6123,7 +6099,6 @@
       <c r="J29" s="6" t="n">
         <v>0.05456852791878172</v>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6162,7 +6137,6 @@
       <c r="J30" s="6" t="n">
         <v>0.1763959390862944</v>
       </c>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6201,7 +6175,6 @@
       <c r="J31" s="6" t="n">
         <v>0.6371613887829073</v>
       </c>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6240,7 +6213,6 @@
       <c r="J32" s="6" t="n">
         <v>0.08383233532934131</v>
       </c>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6279,7 +6251,6 @@
       <c r="J33" s="6" t="n">
         <v>0.7714285714285715</v>
       </c>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6318,7 +6289,6 @@
       <c r="J34" s="6" t="n">
         <v>0.2592592592592592</v>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6357,7 +6327,6 @@
       <c r="J35" s="6" t="n">
         <v>0.8928571428571429</v>
       </c>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6396,7 +6365,6 @@
       <c r="J36" s="6" t="n">
         <v>0.01497005988023952</v>
       </c>
-      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6435,7 +6403,6 @@
       <c r="J37" s="6" t="n">
         <v>0.06467065868263473</v>
       </c>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6474,7 +6441,6 @@
       <c r="J38" s="6" t="n">
         <v>0.6283749790373973</v>
       </c>
-      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6513,7 +6479,6 @@
       <c r="J39" s="6" t="n">
         <v>0.08540165465705898</v>
       </c>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6552,7 +6517,6 @@
       <c r="J40" s="6" t="n">
         <v>0.6921875</v>
       </c>
-      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6591,7 +6555,6 @@
       <c r="J41" s="6" t="n">
         <v>0.2866817155756208</v>
       </c>
-      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6630,7 +6593,6 @@
       <c r="J42" s="6" t="n">
         <v>0.6299212598425197</v>
       </c>
-      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6669,7 +6631,6 @@
       <c r="J43" s="6" t="n">
         <v>0.01067520683213237</v>
       </c>
-      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6708,7 +6669,6 @@
       <c r="J44" s="6" t="n">
         <v>0.05911395783293302</v>
       </c>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6747,7 +6707,6 @@
       <c r="J45" s="6" t="n">
         <v>0.5831545064377682</v>
       </c>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6786,7 +6745,6 @@
       <c r="J46" s="6" t="n">
         <v>0.07359705611775529</v>
       </c>
-      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6825,7 +6783,6 @@
       <c r="J47" s="6" t="n">
         <v>0.65</v>
       </c>
-      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6864,7 +6821,6 @@
       <c r="J48" s="6" t="n">
         <v>0.3846153846153846</v>
       </c>
-      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6903,7 +6859,6 @@
       <c r="J49" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6942,7 +6897,6 @@
       <c r="J50" s="6" t="n">
         <v>0.01655933762649494</v>
       </c>
-      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6981,7 +6935,6 @@
       <c r="J51" s="6" t="n">
         <v>0.04783808647654094</v>
       </c>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -7020,7 +6973,6 @@
       <c r="J52" s="6" t="n">
         <v>0.7168760708166761</v>
       </c>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7059,7 +7011,6 @@
       <c r="J53" s="6" t="n">
         <v>0.08803027285401314</v>
       </c>
-      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7098,7 +7049,6 @@
       <c r="J54" s="6" t="n">
         <v>0.5882352941176471</v>
       </c>
-      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -7137,7 +7087,6 @@
       <c r="J55" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -7176,7 +7125,6 @@
       <c r="J56" s="6" t="n">
         <v>0.6263736263736264</v>
       </c>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -7215,7 +7163,6 @@
       <c r="J57" s="6" t="n">
         <v>0.0113523202549293</v>
       </c>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -7254,7 +7201,6 @@
       <c r="J58" s="6" t="n">
         <v>0.05178251344353715</v>
       </c>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7830,8 +7776,6 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
@@ -8222,6 +8166,1523 @@
       </c>
       <c r="G88" s="6" t="n">
         <v>-0.1364730883470224</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web): origem x device, 01-05/10 vs referências (receita captada GA4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sessões Out</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 03-07/09</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 24-28/09</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos Out</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 24-28/09</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>CVR Out</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>CVR 24-28/09</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 24-28/09</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 03-07/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>google / organic</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2092</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>1570</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>0.00246791707798618</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.00445859872611465</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>-2129.96</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>-3819.019989</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1791</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>1563</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>1673</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.008375209380234505</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.01016138673042439</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>-2053.810003</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>-1592.530006999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bing / organic</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.02272727272727273</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>-1149.979998</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>l.instagram.com / referral</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0.02222222222222222</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.01652892561983471</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>-848.9700059999999</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>598.489999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>google / pmax</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>-799.950002</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>crm / web_push</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>135</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.009259259259259259</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.01481481481481482</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>-744.9700029999999</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>584.989998</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>instagram.com / referral</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>0.03448275862068965</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>-679.989998</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>beacons.ai / referral</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>-594.989997</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>-234.980001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>136</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>138</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0.02205882352941177</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>1746.069998</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>1746.069998</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1362</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.01027900146842878</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.004761904761904762</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>2459.720005000001</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>1675.970001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>7731</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>8910</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>7561</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0.007114215496054844</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.006083851342415025</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>6906.359983999999</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>1770.979993000001</v>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web): origem x device, 01-05/10 vs referências (receita captada GA4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sessões Out</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 03-07/09</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 24-28/09</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos Out</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 24-28/09</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>CVR Out</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>CVR 24-28/09</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 24-28/09</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 03-07/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>linktr.ee / referral</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>161</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0.00909090909090909</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.01333333333333333</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>-480.290004</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>-321.56</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>crm / whatsapp</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>-449.969998</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>bonifiq / SMS</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>-444.749998</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>221</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>87</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0.009009009009009009</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>-439.969999</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>-237.979999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>paquetaesportes.com.br / referral</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.02040816326530612</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>-429.999997</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>119.980002</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>paquetaesportes.com.br / referral</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>147</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>163</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>152</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0.02040816326530612</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>0.01973684210526316</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>-375.9900010000001</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>5.349999000000025</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>google / organic</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>466</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>635</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>632</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.006437768240343348</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.007911392405063292</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>-351.2399999999999</v>
+      </c>
+      <c r="K24" s="5" t="n">
+        <v>-217.4399990000001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>l.facebook.com / referral</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>-209.980002</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>574</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>585</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.01068702290076336</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.008547008547008548</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>1041.309998</v>
+      </c>
+      <c r="K26" s="5" t="n">
+        <v>1540.940002</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>677</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>677</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0.01920236336779911</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>0.01052631578947368</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>1845.510009</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>1499.640002</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>2841</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>4470</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>3175</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0.01583949313621964</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.009763779527559056</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>3066.870015000001</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>3760.300000000002</v>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app): origem x device, 01-05/10 vs referências (receita captada GA4) | App: receita e pedidos de Out com compra duplicada; usar sessões</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Sessões Out</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 03-07/09</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 24-28/09</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos Out</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 24-28/09</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>CVR Out</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>CVR 24-28/09</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 24-28/09</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 03-07/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>google / organic</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>0.1025641025641026</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>-2919.960002</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>3004</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>3002</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>2813</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>0.007323568575233023</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>0.01173124777817277</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>-1875.430001000002</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>1261.45999</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>crm / app_push</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>439</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>983</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>897</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>0.009111617312072893</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>0.01337792642140468</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>-1249.750013</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>-671.3500099999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>eitri-shop-source / (not set)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>-389.859998</v>
+      </c>
+      <c r="K36" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>apps.facebook.com / (not set)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>198</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>188</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>0.007462686567164179</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>-279.96</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>awin / (not set)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>-247.939998</v>
+      </c>
+      <c r="K38" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>firebase / app_push</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>-99.989998</v>
+      </c>
+      <c r="K39" s="5" t="n">
+        <v>-469.9499980000001</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>crm / app_push</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>192</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>243</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0.01351351351351351</v>
+      </c>
+      <c r="J40" s="5" t="n">
+        <v>-64.84999900000003</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <v>314.8599990000001</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>526</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>478</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>0.03611738148984198</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>0.03765690376569038</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>3454.870006999998</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>8468.000006999997</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>(not set)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>0.3255813953488372</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0.04838709677419355</v>
+      </c>
+      <c r="J42" s="5" t="n">
+        <v>5770.110009</v>
+      </c>
+      <c r="K42" s="5" t="n">
+        <v>5065.200014</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>1564</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>1411</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>1338</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>0.03836317135549872</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0.0343796711509716</v>
+      </c>
+      <c r="J43" s="5" t="n">
+        <v>12881.139985</v>
+      </c>
+      <c r="K43" s="5" t="n">
+        <v>17168.529984</v>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Oscar web: origem e funil de outubro dependem de nova extração com o filtro atualizado (o export atual de outubro ainda tem bots no desktop).</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh workbook with new Oscar web October extraction
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iFLn21AiUGfBb2WhkxcsV
</commit_message>
<xml_diff>
--- a/analise/Respostas_por_bandeira_set26.xlsx
+++ b/analise/Respostas_por_bandeira_set26.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Diadora: -R$ 22.892 (43,8% da meta). Em R$, entre as bandeiras do Grupo: Oscar web -R$ 21.391 (75,3%), App -R$ 17.068 (67,0%), Esportes -R$ 4.848 (91,4%); Calçados +R$ 6.388 (129,5%). Grupo (4 bandeiras) -R$ 36.918 (83,0%). Faturado ainda amadurece.</t>
+          <t>Diadora: -R$ 22.892 (43,8% da meta). Em R$, entre as bandeiras do Grupo: Oscar web -R$ 21.391 (75,3%), App -R$ 17.069 (67,0%), Esportes -R$ 4.848 (91,4%); Calçados +R$ 6.388 (129,5%). Grupo (4 bandeiras) -R$ 36.841 (83,0%). Faturado ainda amadurece.</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -709,16 +709,16 @@
         <v>202605</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>318371</v>
+        <v>318584</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.009611428176561307</v>
+        <v>0.009501418778093062</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>344.4644727720828</v>
+        <v>350.6384514182847</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>1054061.286682573</v>
+        <v>1061382.592443148</v>
       </c>
     </row>
     <row r="4">
@@ -731,16 +731,16 @@
         <v>202606</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>303083</v>
+        <v>302886</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.01072973409924014</v>
+        <v>0.01064426880080294</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>360.1643693967197</v>
+        <v>367.7144788566365</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>1171254.529278133</v>
+        <v>1185511.479833796</v>
       </c>
     </row>
     <row r="5">
@@ -753,16 +753,16 @@
         <v>202607</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>343990</v>
+        <v>344514</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.01287246722288439</v>
+        <v>0.01269904851471929</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>394.1893495229506</v>
+        <v>401.0144010982897</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1745470.439687625</v>
+        <v>1754438.004805017</v>
       </c>
     </row>
     <row r="6">
@@ -775,16 +775,16 @@
         <v>202608</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>280282</v>
+        <v>281568</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.01132430908870352</v>
+        <v>0.01107015001704739</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>332.0564378973676</v>
+        <v>337.6660344742969</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1053947.133886245</v>
+        <v>1052505.029456384</v>
       </c>
     </row>
     <row r="7">
@@ -797,16 +797,16 @@
         <v>202609</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>247080</v>
+        <v>245193</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.009713453132588635</v>
+        <v>0.009506796686691708</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>352.7904436360002</v>
+        <v>357.483778684379</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>846697.0647264005</v>
+        <v>833294.6881132874</v>
       </c>
     </row>
     <row r="8">
@@ -819,16 +819,16 @@
         <v>202610</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>32037</v>
+        <v>29066</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.01030058994287855</v>
+        <v>0.01238560517443061</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>367.634362366622</v>
+        <v>372.9152228734548</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>121319.3395809853</v>
+        <v>134249.4802344437</v>
       </c>
     </row>
     <row r="9">
@@ -1701,7 +1701,7 @@
         <v>265721</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>188936</v>
+        <v>188929</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3171</v>
@@ -1736,7 +1736,7 @@
         <v>58118</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>36179</v>
+        <v>36172</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>1567</v>
@@ -1777,13 +1777,13 @@
         <v>1598</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>518071.3098940001</v>
+        <v>518071.3098939999</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>0.007722045037208853</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>324.199818456821</v>
+        <v>324.1998184568209</v>
       </c>
     </row>
     <row r="6">
@@ -1838,10 +1838,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>248790</v>
+        <v>247187</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>178701</v>
+        <v>176550</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>2521</v>
@@ -1850,7 +1850,7 @@
         <v>887772.7301079999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.01013304393263395</v>
+        <v>0.01019875640709261</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>352.1510234462514</v>
@@ -1873,10 +1873,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>49658</v>
+        <v>48055</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>30798</v>
+        <v>28647</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1384</v>
@@ -1885,7 +1885,7 @@
         <v>503337.839989</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.02787063514438761</v>
+        <v>0.02880033295182603</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>363.6834103966763</v>
@@ -1917,13 +1917,13 @@
         <v>1135</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>383624.910121</v>
+        <v>383624.9101209999</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>0.005725989940419435</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>337.9955155251101</v>
+        <v>337.99551552511</v>
       </c>
     </row>
     <row r="10">
@@ -1978,22 +1978,22 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>29882</v>
+        <v>29957</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>25582</v>
+        <v>25483</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>142584.533237606</v>
+        <v>150556.7818969148</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.01184659661334583</v>
+        <v>0.01185031879026605</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>402.78116733787</v>
+        <v>424.1036109772248</v>
       </c>
     </row>
     <row r="12">
@@ -2013,22 +2013,22 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>7120</v>
+        <v>6886</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5667</v>
+        <v>5410</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>82379.71769027352</v>
+        <v>86864.53313560033</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.03019662921348315</v>
+        <v>0.03194888178913738</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>383.1614776291792</v>
+        <v>394.8387869800015</v>
       </c>
     </row>
     <row r="13">
@@ -2048,22 +2048,22 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22690</v>
+        <v>22999</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>19850</v>
+        <v>20008</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>60026.41962002258</v>
+        <v>63500.20780777142</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0.006081974438078449</v>
+        <v>0.005826340275664159</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>434.9740552175549</v>
+        <v>473.8821478191897</v>
       </c>
     </row>
     <row r="14">
@@ -2092,13 +2092,13 @@
         <v>1</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>178.3959273098884</v>
+        <v>192.040953543025</v>
       </c>
       <c r="H14" s="4" t="n">
         <v>0.01388888888888889</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>178.3959273098884</v>
+        <v>192.040953543025</v>
       </c>
     </row>
     <row r="15">
@@ -2256,10 +2256,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>35799</v>
+        <v>35791</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>29390</v>
+        <v>29387</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>396</v>
@@ -2268,10 +2268,10 @@
         <v>133941.499986</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.01106176150171793</v>
+        <v>0.01106423402531363</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>338.2361110757576</v>
+        <v>338.2361110757577</v>
       </c>
     </row>
     <row r="20">
@@ -2291,22 +2291,22 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>7394</v>
+        <v>7386</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>5025</v>
+        <v>5022</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>222</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>79800.85997600001</v>
+        <v>79800.85997600004</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.03002434406275358</v>
+        <v>0.03005686433793664</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>359.4633332252253</v>
+        <v>359.4633332252254</v>
       </c>
     </row>
     <row r="21">
@@ -4998,7 +4998,7 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -5086,25 +5086,25 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.640110978993262</v>
+        <v>0.6402378592666006</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>0.67665719384046</v>
+        <v>0.655596643436211</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>3.6546214847198</v>
+        <v>1.535878416961045</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>0.05709356040834712</v>
+        <v>0.02398918456213139</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>0.4624340549390576</v>
+        <v>0.4357875116495806</v>
       </c>
       <c r="I3" s="6" t="n">
         <v>0.6356011183597391</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>0.58650132140679</v>
+        <v>0.5868592351505288</v>
       </c>
     </row>
     <row r="4">
@@ -5127,16 +5127,16 @@
         <v>0.09044670499778859</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.1024564145138448</v>
+        <v>0.08748237335936652</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1.20097095160562</v>
+        <v>-0.2964331638422066</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.1327821673144405</v>
+        <v>-0.03277434637883758</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.08693941778127459</v>
+        <v>0.08554319931565441</v>
       </c>
       <c r="I4" s="6" t="n">
         <v>0.08357771260997067</v>
@@ -5165,16 +5165,16 @@
         <v>0.7799511002444988</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.8317445185891325</v>
+        <v>0.7823930564166151</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>5.179341834463369</v>
+        <v>0.2441956172116289</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.06640598151396615</v>
+        <v>0.003130909324124076</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>0.6515837104072398</v>
+        <v>0.655</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>0.793859649122807</v>
@@ -5203,16 +5203,16 @@
         <v>0.6858934169278997</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.5249283667621777</v>
+        <v>0.7258320126782885</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>-16.09650501657221</v>
+        <v>3.993859575038872</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>-0.2346793921520354</v>
+        <v>0.05822857424302552</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>1.319444444444444</v>
+        <v>1.450381679389313</v>
       </c>
       <c r="I6" s="6" t="n">
         <v>0.9171270718232044</v>
@@ -5255,7 +5255,7 @@
         <v>0.01797196702211856</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.9157894736842105</v>
+        <v>0.9315789473684211</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>0.963855421686747</v>
@@ -5284,16 +5284,16 @@
         <v>0.04343210968597966</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.04087512819260634</v>
+        <v>0.04539537910836317</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>-0.2556981493373321</v>
+        <v>0.1963269422383507</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>-0.05887306676697635</v>
+        <v>0.04520317885956326</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.06845003933910307</v>
+        <v>0.07570573139435414</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>0.05865102639296188</v>
@@ -5322,16 +5322,16 @@
         <v>0.07054400707651481</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.08521756116618645</v>
+        <v>0.06844560147521424</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.467355408967164</v>
+        <v>-0.2098405601300576</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.2080056789764737</v>
+        <v>-0.02974605056138313</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.05664830841856806</v>
+        <v>0.05603079555175364</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>0.06634897360703812</v>
@@ -5369,7 +5369,7 @@
         <v>-0.05050426151838094</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>0.6750922887612797</v>
+        <v>0.6654299323138632</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0.6928712990210798</v>
@@ -5407,7 +5407,7 @@
         <v>-0.2138743429198724</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>0.0657704868231184</v>
+        <v>0.06615430982519591</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>0.05642714743867557</v>
@@ -5445,7 +5445,7 @@
         <v>-0.06338785918469547</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.4919168591224019</v>
+        <v>0.5</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0.6359447004608295</v>
@@ -5483,7 +5483,7 @@
         <v>0.05366608434841291</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.5328638497652582</v>
+        <v>0.5353075170842825</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>0.3514492753623188</v>
@@ -5521,7 +5521,7 @@
         <v>-0.02409881890093135</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.7004405286343612</v>
+        <v>0.7106382978723405</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>0.6494845360824743</v>
@@ -5559,7 +5559,7 @@
         <v>-0.2428871827421585</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.01207564365459102</v>
+        <v>0.01258288125376733</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>0.008191037531420647</v>
@@ -5597,7 +5597,7 @@
         <v>-0.2637051653723438</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.03235361130097972</v>
+        <v>0.03307715491259795</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>0.0358845453757476</v>
@@ -7837,16 +7837,16 @@
         </is>
       </c>
       <c r="D77" s="6" t="n">
-        <v>0.6448324220411894</v>
+        <v>0.6449035552193646</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>0.6644046992810801</v>
+        <v>0.6531370691539751</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>1.957227723989075</v>
+        <v>0.823351393461047</v>
       </c>
       <c r="G77" s="6" t="n">
-        <v>0.03035250178323157</v>
+        <v>0.01276704689867914</v>
       </c>
     </row>
     <row r="78">
@@ -7869,13 +7869,13 @@
         <v>0.07919751728856633</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>0.08606265340054367</v>
+        <v>0.07742943210978467</v>
       </c>
       <c r="F78" s="7" t="n">
-        <v>0.6865136111977338</v>
+        <v>-0.1768085178781659</v>
       </c>
       <c r="G78" s="6" t="n">
-        <v>0.08668372882148989</v>
+        <v>-0.02232500764309842</v>
       </c>
     </row>
     <row r="79">
@@ -7898,13 +7898,13 @@
         <v>0.7701326751002777</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>0.7865685372585096</v>
+        <v>0.75</v>
       </c>
       <c r="F79" s="7" t="n">
-        <v>1.64358621582319</v>
+        <v>-2.013267510027772</v>
       </c>
       <c r="G79" s="6" t="n">
-        <v>0.0213415982591465</v>
+        <v>-0.02614182692307698</v>
       </c>
     </row>
     <row r="80">
@@ -7927,13 +7927,13 @@
         <v>0.5949519230769231</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>0.4826510721247563</v>
+        <v>0.5946205571565802</v>
       </c>
       <c r="F80" s="7" t="n">
-        <v>-11.23008509521668</v>
+        <v>-0.03313659203428854</v>
       </c>
       <c r="G80" s="6" t="n">
-        <v>-0.1887561777620258</v>
+        <v>-0.0005569625166167436</v>
       </c>
     </row>
     <row r="81">
@@ -7985,13 +7985,13 @@
         <v>0.03157148791633067</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>0.02881950859043044</v>
+        <v>0.03045855182416602</v>
       </c>
       <c r="F82" s="7" t="n">
-        <v>-0.2751979325900222</v>
+        <v>-0.1112936092164649</v>
       </c>
       <c r="G82" s="6" t="n">
-        <v>-0.08716660213143557</v>
+        <v>-0.03525130317310676</v>
       </c>
     </row>
     <row r="83">
@@ -8179,7 +8179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -8189,16 +8189,17 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Paquetá Esportes (web): origem x device, 01-05/10 vs referências (receita captada GA4)</t>
+          <t>Oscar Calçados (web): origem x device, 01-05/10 vs referências (receita captada GA4) | Web: direto desktop de Out ainda tem cerca de 1,5 mil sessões de resíduo (pedidos são reais)</t>
         </is>
       </c>
     </row>
@@ -8235,25 +8236,30 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Pedidos 03-07/09</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Pedidos 24-28/09</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>CVR Out</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>CVR 24-28/09</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>dRec vs 24-28/09</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>dRec vs 03-07/09</t>
         </is>
@@ -8262,7 +8268,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>google / organic</t>
+          <t>google / cpc</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8271,31 +8277,34 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2026</v>
+        <v>10537</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2092</v>
+        <v>18176</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1570</v>
+        <v>13555</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>0.00246791707798618</v>
+        <v>72</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>64</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.00445859872611465</v>
-      </c>
-      <c r="J3" s="5" t="n">
-        <v>-2129.96</v>
+        <v>0.002752206510391952</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0.004721504979712283</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-3819.019989</v>
+        <v>-6664.843679511983</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>-6433.363660511985</v>
       </c>
     </row>
     <row r="4">
@@ -8310,115 +8319,124 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1791</v>
+        <v>1452</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1563</v>
+        <v>2227</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1673</v>
+        <v>2178</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>0.008375209380234505</v>
+        <v>63</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>68</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>0.01016138673042439</v>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>-2053.810003</v>
+        <v>0.03099173553719008</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.03122130394857667</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-1592.530006999999</v>
+        <v>-6242.8731032826</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>-5161.403098282593</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bing / organic</t>
+          <t>cariocacalcados.com.br / referral</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>28</v>
+        <v>247</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>40</v>
+        <v>327</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>44</v>
+        <v>300</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.02272727272727273</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>-1149.979998</v>
+        <v>0</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>0.01</v>
       </c>
       <c r="K5" s="5" t="n">
+        <v>-1869.959997</v>
+      </c>
+      <c r="L5" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>l.instagram.com / referral</t>
+          <t>cariocacalcados.com.br / referral</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>44</v>
+        <v>114</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>242</v>
+        <v>132</v>
       </c>
       <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0.02222222222222222</v>
-      </c>
       <c r="I6" s="4" t="n">
-        <v>0.01652892561983471</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>-848.9700059999999</v>
+        <v>0</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0.007575757575757576</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>598.489999</v>
+        <v>-1845.889999</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>google / pmax</t>
+          <t>bonifiq / SMS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8427,76 +8445,82 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D7" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I7" s="4" t="n">
-        <v>0.08333333333333333</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>-799.950002</v>
+        <v>0</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0.1</v>
       </c>
       <c r="K7" s="5" t="n">
+        <v>-1017.080002</v>
+      </c>
+      <c r="L7" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>crm / web_push</t>
+          <t>inngage_push / onsite_push</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>108</v>
+        <v>26</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>135</v>
+        <v>82</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>0.009259259259259259</v>
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.01481481481481482</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>-744.9700029999999</v>
+        <v>0</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.03658536585365853</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>584.989998</v>
+        <v>-991.14</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>instagram.com / referral</t>
+          <t>(not set)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8505,298 +8529,321 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>3</v>
+        <v>609</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>7</v>
+        <v>1264</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>29</v>
+        <v>1071</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.03448275862068965</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>-679.989998</v>
+        <v>0</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>0.004668534080298786</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0</v>
+        <v>-923.0599990000001</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>-1987.510003</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>beacons.ai / referral</t>
+          <t>ntp.msn.com / referral</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0</v>
+      <c r="H10" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>-594.989997</v>
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.1111111111111111</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-234.980001</v>
+        <v>-718.48</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>-932.46</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>(direct) / (none)</t>
+          <t>google / organic</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>136</v>
+        <v>4310</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>111</v>
+        <v>5642</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>138</v>
+        <v>5058</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>0.02205882352941177</v>
+        <v>36</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>29</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>1746.069998</v>
+        <v>0.007192575406032482</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>0.005733491498616054</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>1746.069998</v>
+        <v>5255.051704976753</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>-2110.098310023246</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>(direct) / (none)</t>
+          <t>crm / web_push</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1362</v>
+        <v>272</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>720</v>
+        <v>343</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>1890</v>
+        <v>303</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>0.01027900146842878</v>
+        <v>19</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>11</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>0.004761904761904762</v>
-      </c>
-      <c r="J12" s="5" t="n">
-        <v>2459.720005000001</v>
+        <v>0.1102941176470588</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0.03630363036303631</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1675.970001</v>
+        <v>6606.576998513947</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>4489.347000513947</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>google / cpc</t>
+          <t>(direct) / (none)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>2414</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>796</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>1257</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>0.04432477216238608</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>0.07159904534606205</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>8800.547034558862</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>8744.957026558863</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>mobile</t>
         </is>
       </c>
-      <c r="C13" s="3" t="n">
-        <v>7731</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>8910</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>7561</v>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>55</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>0.007114215496054844</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>0.006083851342415025</v>
-      </c>
-      <c r="J13" s="5" t="n">
-        <v>6906.359983999999</v>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>1770.979993000001</v>
-      </c>
-    </row>
-    <row r="14"/>
+      <c r="C14" s="3" t="n">
+        <v>4027</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>8539</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>4341</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.01564440029798858</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0.0129002533978346</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>11842.27878525751</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>6494.538780257517</v>
+      </c>
+    </row>
     <row r="15"/>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Paquetá Calçados (web): origem x device, 01-05/10 vs referências (receita captada GA4)</t>
-        </is>
-      </c>
-    </row>
+    <row r="16"/>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Paquetá Esportes (web): origem x device, 01-05/10 vs referências (receita captada GA4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Origem</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sessões Out</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Sessões 03-07/09</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Sessões 24-28/09</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Pedidos Out</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 03-07/09</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Pedidos 24-28/09</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>CVR Out</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>CVR 24-28/09</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>dRec vs 24-28/09</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>dRec vs 03-07/09</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>linktr.ee / referral</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>mobile</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>161</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>0.00909090909090909</v>
-      </c>
-      <c r="I18" s="4" t="n">
-        <v>0.01333333333333333</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>-480.290004</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>-321.56</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>crm / whatsapp</t>
+          <t>google / organic</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8805,76 +8852,82 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>8</v>
+        <v>2026</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1</v>
+        <v>2092</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>4</v>
+        <v>1570</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="4" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>7</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="J19" s="5" t="n">
-        <v>-449.969998</v>
+        <v>0.00246791707798618</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>0.00445859872611465</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>0</v>
+        <v>-2129.96</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>-3819.019989</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bonifiq / SMS</t>
+          <t>google / cpc</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>mobile</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>6</v>
+        <v>1791</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>30</v>
+        <v>1563</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>11</v>
+        <v>1673</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>17</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>0.09090909090909091</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <v>-444.749998</v>
+        <v>0.008375209380234505</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0.01016138673042439</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>0</v>
+        <v>-2053.810003</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>-1592.530006999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>(direct) / (none)</t>
+          <t>bing / organic</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8883,76 +8936,82 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>221</v>
+        <v>28</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>222</v>
+        <v>44</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>0.009009009009009009</v>
-      </c>
-      <c r="J21" s="5" t="n">
-        <v>-439.969999</v>
+        <v>0</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0.02272727272727273</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-237.979999</v>
+        <v>-1149.979998</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>paquetaesportes.com.br / referral</t>
+          <t>l.instagram.com / referral</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>desktop</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>64</v>
+        <v>242</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>0.02040816326530612</v>
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>0.03125</v>
-      </c>
-      <c r="J22" s="5" t="n">
-        <v>-429.999997</v>
+        <v>0.02222222222222222</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0.01652892561983471</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>119.980002</v>
+        <v>-848.9700059999999</v>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>598.489999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>paquetaesportes.com.br / referral</t>
+          <t>google / pmax</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -8961,37 +9020,40 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>147</v>
+        <v>24</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>163</v>
+        <v>2</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>152</v>
+        <v>12</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="4" t="n">
-        <v>0.02040816326530612</v>
+        <v>0</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>0.01973684210526316</v>
-      </c>
-      <c r="J23" s="5" t="n">
-        <v>-375.9900010000001</v>
+        <v>0</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>0.08333333333333333</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>5.349999000000025</v>
+        <v>-799.950002</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>google / organic</t>
+          <t>crm / web_push</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9000,37 +9062,40 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>466</v>
+        <v>108</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>635</v>
+        <v>80</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>632</v>
+        <v>135</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>0.006437768240343348</v>
+        <v>0</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>0.007911392405063292</v>
-      </c>
-      <c r="J24" s="5" t="n">
-        <v>-351.2399999999999</v>
+        <v>0.009259259259259259</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0.01481481481481482</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>-217.4399990000001</v>
+        <v>-744.9700029999999</v>
+      </c>
+      <c r="L24" s="5" t="n">
+        <v>584.989998</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>l.facebook.com / referral</t>
+          <t>instagram.com / referral</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9042,34 +9107,37 @@
         <v>3</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I25" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="J25" s="5" t="n">
-        <v>-209.980002</v>
+        <v>0</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>0.03448275862068965</v>
       </c>
       <c r="K25" s="5" t="n">
+        <v>-679.989998</v>
+      </c>
+      <c r="L25" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>(direct) / (none)</t>
+          <t>beacons.ai / referral</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9078,37 +9146,40 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>655</v>
+        <v>3</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>574</v>
+        <v>3</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>585</v>
+        <v>8</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>0.01068702290076336</v>
+        <v>1</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I26" s="4" t="n">
-        <v>0.008547008547008548</v>
-      </c>
-      <c r="J26" s="5" t="n">
-        <v>1041.309998</v>
+        <v>0</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>0.125</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>1540.940002</v>
+        <v>-594.989997</v>
+      </c>
+      <c r="L26" s="5" t="n">
+        <v>-234.980001</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>google / cpc</t>
+          <t>(data not available)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9117,572 +9188,1308 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>677</v>
+        <v>33</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>677</v>
+        <v>20</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>760</v>
+        <v>18</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="H27" s="4" t="n">
-        <v>0.01920236336779911</v>
+        <v>0</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>0.01052631578947368</v>
-      </c>
-      <c r="J27" s="5" t="n">
-        <v>1845.510009</v>
+        <v>0.06060606060606061</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>1499.640002</v>
+        <v>1532.45</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>1532.45</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>136</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>138</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.02205882352941177</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>1746.069998</v>
+      </c>
+      <c r="L28" s="5" t="n">
+        <v>1746.069998</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>1362</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>0.01027900146842878</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>0.004761904761904762</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>2459.720005000001</v>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>1675.970001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>google / cpc</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>mobile</t>
         </is>
       </c>
-      <c r="C28" s="3" t="n">
-        <v>2841</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>4470</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>3175</v>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="G28" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>0.01583949313621964</v>
-      </c>
-      <c r="I28" s="4" t="n">
-        <v>0.009763779527559056</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>3066.870015000001</v>
-      </c>
-      <c r="K28" s="5" t="n">
-        <v>3760.300000000002</v>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>Oscar Calçados (app): origem x device, 01-05/10 vs referências (receita captada GA4) | App: receita e pedidos de Out com compra duplicada; usar sessões</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="C30" s="3" t="n">
+        <v>7731</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>8910</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>7561</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0.007114215496054844</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>0.006083851342415025</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>6906.359983999999</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>1770.979993000001</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Paquetá Calçados (web): origem x device, 01-05/10 vs referências (receita captada GA4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Origem</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Device</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Sessões Out</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Sessões 03-07/09</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Sessões 24-28/09</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Pedidos Out</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 03-07/09</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Pedidos 24-28/09</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>CVR Out</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>CVR 24-28/09</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>dRec vs 24-28/09</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>dRec vs 03-07/09</t>
         </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>google / organic</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>iOS</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="D33" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>39</v>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>0.1025641025641026</v>
-      </c>
-      <c r="J33" s="5" t="n">
-        <v>-2919.960002</v>
-      </c>
-      <c r="K33" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>(direct) / (none)</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Android</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="n">
-        <v>3004</v>
-      </c>
-      <c r="D34" s="3" t="n">
-        <v>3002</v>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>2813</v>
-      </c>
-      <c r="F34" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="G34" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="H34" s="4" t="n">
-        <v>0.007323568575233023</v>
-      </c>
-      <c r="I34" s="4" t="n">
-        <v>0.01173124777817277</v>
-      </c>
-      <c r="J34" s="5" t="n">
-        <v>-1875.430001000002</v>
-      </c>
-      <c r="K34" s="5" t="n">
-        <v>1261.45999</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>crm / app_push</t>
+          <t>linktr.ee / referral</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>439</v>
+        <v>110</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>983</v>
+        <v>161</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>897</v>
+        <v>150</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="H35" s="4" t="n">
-        <v>0.009111617312072893</v>
+        <v>1</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>0.01337792642140468</v>
-      </c>
-      <c r="J35" s="5" t="n">
-        <v>-1249.750013</v>
+        <v>0.00909090909090909</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>0.01333333333333333</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>-671.3500099999999</v>
+        <v>-480.290004</v>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>-321.56</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>eitri-shop-source / (not set)</t>
+          <t>crm / whatsapp</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>iOS</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H36" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I36" s="4" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="J36" s="5" t="n">
-        <v>-389.859998</v>
+        <v>0</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>0.25</v>
       </c>
       <c r="K36" s="5" t="n">
+        <v>-449.969998</v>
+      </c>
+      <c r="L36" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>apps.facebook.com / (not set)</t>
+          <t>bonifiq / SMS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>198</v>
+        <v>6</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>188</v>
+        <v>30</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>268</v>
+        <v>11</v>
       </c>
       <c r="F37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H37" s="4" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>0.007462686567164179</v>
-      </c>
-      <c r="J37" s="5" t="n">
-        <v>-279.96</v>
+        <v>0</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>0.09090909090909091</v>
       </c>
       <c r="K37" s="5" t="n">
+        <v>-444.749998</v>
+      </c>
+      <c r="L37" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>awin / (not set)</t>
+          <t>(direct) / (none)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="D38" s="3" t="n">
+        <v>87</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="H38" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F38" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" s="4" t="n"/>
       <c r="I38" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J38" s="5" t="n">
-        <v>-247.939998</v>
+        <v>0</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>0.009009009009009009</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>0</v>
+        <v>-439.969999</v>
+      </c>
+      <c r="L38" s="5" t="n">
+        <v>-237.979999</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>firebase / app_push</t>
+          <t>paquetaesportes.com.br / referral</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>iOS</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" s="4" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>0.05263157894736842</v>
-      </c>
-      <c r="J39" s="5" t="n">
-        <v>-99.989998</v>
+        <v>0.02040816326530612</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>0.03125</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>-469.9499980000001</v>
+        <v>-429.999997</v>
+      </c>
+      <c r="L39" s="5" t="n">
+        <v>119.980002</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>crm / app_push</t>
+          <t>paquetaesportes.com.br / referral</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>iOS</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>192</v>
+        <v>147</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>243</v>
+        <v>163</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>222</v>
+        <v>152</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G40" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H40" s="4" t="n">
-        <v>0.03125</v>
+      <c r="H40" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="I40" s="4" t="n">
-        <v>0.01351351351351351</v>
-      </c>
-      <c r="J40" s="5" t="n">
-        <v>-64.84999900000003</v>
+        <v>0.02040816326530612</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>0.01973684210526316</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>314.8599990000001</v>
+        <v>-375.9900010000001</v>
+      </c>
+      <c r="L40" s="5" t="n">
+        <v>5.349999000000025</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>google / cpc</t>
+          <t>google / organic</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>iOS</t>
+          <t>desktop</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>443</v>
+        <v>466</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>526</v>
+        <v>635</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>478</v>
+        <v>632</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>0.03611738148984198</v>
+        <v>5</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>0.03765690376569038</v>
-      </c>
-      <c r="J41" s="5" t="n">
-        <v>3454.870006999998</v>
+        <v>0.006437768240343348</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>0.007911392405063292</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>8468.000006999997</v>
+        <v>-351.2399999999999</v>
+      </c>
+      <c r="L41" s="5" t="n">
+        <v>-217.4399990000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>(not set)</t>
+          <t>l.facebook.com / referral</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>iOS</t>
+          <t>mobile</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>0.3255813953488372</v>
+        <v>0</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0.04838709677419355</v>
-      </c>
-      <c r="J42" s="5" t="n">
-        <v>5770.110009</v>
+        <v>0</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>0.25</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>5065.200014</v>
+        <v>-209.980002</v>
+      </c>
+      <c r="L42" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Meta Ads (soma das grafias)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>1582</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>1615</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>1508</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0.004424778761061947</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>0.003315649867374005</v>
+      </c>
+      <c r="K43" s="5" t="n">
+        <v>992.8900039999999</v>
+      </c>
+      <c r="L43" s="5" t="n">
+        <v>-155.0699970000001</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>(direct) / (none)</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>iOS</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="n">
-        <v>1564</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>1411</v>
-      </c>
-      <c r="E43" s="3" t="n">
-        <v>1338</v>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>60</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>0.03836317135549872</v>
-      </c>
-      <c r="I43" s="4" t="n">
-        <v>0.0343796711509716</v>
-      </c>
-      <c r="J43" s="5" t="n">
-        <v>12881.139985</v>
-      </c>
-      <c r="K43" s="5" t="n">
-        <v>17168.529984</v>
-      </c>
-    </row>
-    <row r="44"/>
-    <row r="45"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>574</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>585</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0.01068702290076336</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>0.008547008547008548</v>
+      </c>
+      <c r="K44" s="5" t="n">
+        <v>1041.309998</v>
+      </c>
+      <c r="L44" s="5" t="n">
+        <v>1540.940002</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>677</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>677</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>0.01920236336779911</v>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>0.01052631578947368</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>1845.510009</v>
+      </c>
+      <c r="L45" s="5" t="n">
+        <v>1499.640002</v>
+      </c>
+    </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Oscar web: origem e funil de outubro dependem de nova extração com o filtro atualizado (o export atual de outubro ainda tem bots no desktop).</t>
-        </is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>mobile</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>2841</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>4470</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>3175</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>0.01583949313621964</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>0.009763779527559056</v>
+      </c>
+      <c r="K46" s="5" t="n">
+        <v>3066.870015000001</v>
+      </c>
+      <c r="L46" s="5" t="n">
+        <v>3760.300000000002</v>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>Oscar Calçados (app): origem x device, 01-05/10 vs referências (receita captada GA4) | App: receita e pedidos de Out com compra duplicada; usar sessões</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Origem</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Sessões Out</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 03-07/09</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Sessões 24-28/09</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos Out</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 03-07/09</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Pedidos 24-28/09</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>CVR Out</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>CVR 24-28/09</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 24-28/09</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>dRec vs 03-07/09</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>google / organic</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>0.1025641025641026</v>
+      </c>
+      <c r="K51" s="5" t="n">
+        <v>-2919.960002</v>
+      </c>
+      <c r="L51" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="n">
+        <v>3004</v>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>3002</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>2813</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>0.007323568575233023</v>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>0.01173124777817277</v>
+      </c>
+      <c r="K52" s="5" t="n">
+        <v>-1875.430001000002</v>
+      </c>
+      <c r="L52" s="5" t="n">
+        <v>1261.45999</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>crm / app_push</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="n">
+        <v>439</v>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>983</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>897</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>0.009111617312072893</v>
+      </c>
+      <c r="J53" s="4" t="n">
+        <v>0.01337792642140468</v>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>-1249.750013</v>
+      </c>
+      <c r="L53" s="5" t="n">
+        <v>-671.3500099999999</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>eitri-shop-source / (not set)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="4" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="K54" s="5" t="n">
+        <v>-389.859998</v>
+      </c>
+      <c r="L54" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>apps.facebook.com / (not set)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="n">
+        <v>198</v>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>188</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>0.007462686567164179</v>
+      </c>
+      <c r="K55" s="5" t="n">
+        <v>-279.96</v>
+      </c>
+      <c r="L55" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>awin / (not set)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I56" s="4" t="n"/>
+      <c r="J56" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="5" t="n">
+        <v>-247.939998</v>
+      </c>
+      <c r="L56" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>firebase / app_push</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4" t="n">
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="K57" s="5" t="n">
+        <v>-99.989998</v>
+      </c>
+      <c r="L57" s="5" t="n">
+        <v>-469.9499980000001</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>crm / app_push</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="n">
+        <v>192</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>243</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>0.01351351351351351</v>
+      </c>
+      <c r="K58" s="5" t="n">
+        <v>-64.84999900000003</v>
+      </c>
+      <c r="L58" s="5" t="n">
+        <v>314.8599990000001</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>(not set)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>157</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>126</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>0.2522522522522522</v>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>0.253968253968254</v>
+      </c>
+      <c r="K59" s="5" t="n">
+        <v>1320.18001</v>
+      </c>
+      <c r="L59" s="5" t="n">
+        <v>8050.979995999999</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>google / cpc</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n">
+        <v>443</v>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>526</v>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>478</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>0.03611738148984198</v>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>0.03765690376569038</v>
+      </c>
+      <c r="K60" s="5" t="n">
+        <v>3454.870006999998</v>
+      </c>
+      <c r="L60" s="5" t="n">
+        <v>8468.000006999997</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>(not set)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>0.3255813953488372</v>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>0.04838709677419355</v>
+      </c>
+      <c r="K61" s="5" t="n">
+        <v>5770.110009</v>
+      </c>
+      <c r="L61" s="5" t="n">
+        <v>5065.200014</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>(direct) / (none)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>iOS</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="n">
+        <v>1564</v>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>1411</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>1338</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>0.03836317135549872</v>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>0.0343796711509716</v>
+      </c>
+      <c r="K62" s="5" t="n">
+        <v>12881.139985</v>
+      </c>
+      <c r="L62" s="5" t="n">
+        <v>17168.529984</v>
       </c>
     </row>
   </sheetData>
@@ -9834,16 +10641,16 @@
         <v>265721</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>248790</v>
+        <v>247187</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-0.06371720714584095</v>
+        <v>-0.06974985040700588</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0.01193356942055765</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.01013304393263395</v>
+        <v>0.01019875640709261</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>338.7555628684958</v>
@@ -9873,16 +10680,16 @@
         <v>-207184</v>
       </c>
       <c r="P3" s="5" t="n">
-        <v>-45456.11044667152</v>
+        <v>-49759.8222797596</v>
       </c>
       <c r="Q3" s="5" t="n">
-        <v>-100779.3357848012</v>
+        <v>-96475.62395171315</v>
       </c>
       <c r="R3" s="5" t="n">
-        <v>22427.62875571817</v>
+        <v>22427.62875571827</v>
       </c>
       <c r="S3" s="5" t="n">
-        <v>-83376.18252424549</v>
+        <v>-83376.1825242456</v>
       </c>
     </row>
     <row r="4">
@@ -10271,13 +11078,13 @@
         <v>465538</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>502872</v>
+        <v>501269</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>0.013</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.009107413209396047</v>
+        <v>0.009136537658294069</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>300</v>
@@ -10292,10 +11099,10 @@
         <v>1237130.99</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>145602.6</v>
+        <v>139350.9</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-587241.8713693772</v>
+        <v>-580990.1713693771</v>
       </c>
       <c r="L3" s="5" t="n">
         <v>244257.2450402343</v>
@@ -10461,16 +11268,16 @@
         <v>58118</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>49658</v>
+        <v>48055</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-0.1455659176158849</v>
+        <v>-0.1731477339206442</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0.02696238686809594</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.02787063514438761</v>
+        <v>0.02880033295182603</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>353.8999872099554</v>
@@ -10485,10 +11292,10 @@
         <v>503337.8399890001</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-80725.22159132594</v>
+        <v>-96021.02894485969</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>15961.52393190408</v>
+        <v>31257.33128543783</v>
       </c>
       <c r="M3" s="5" t="n">
         <v>13540.25769042178</v>
@@ -10516,16 +11323,16 @@
         <v>0.005725989940419435</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>324.199818456821</v>
+        <v>324.1998184568209</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>337.9955155251101</v>
+        <v>337.99551552511</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>518071.3098940001</v>
+        <v>518071.3098939998</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>383624.910121</v>
+        <v>383624.9101209998</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>-21832.89791043575</v>
@@ -10534,7 +11341,7 @@
         <v>-128271.6180350724</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>15658.11617250805</v>
+        <v>15658.11617250811</v>
       </c>
     </row>
     <row r="5">
@@ -10682,13 +11489,13 @@
         <v>0.4623795997693441</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>264189.8699629999</v>
+        <v>264189.8699630001</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>135106.590022</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>-129083.2799409999</v>
+        <v>-129083.2799410001</v>
       </c>
     </row>
     <row r="11">
@@ -10772,7 +11579,7 @@
         <v>8080.720001</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>-8558.620000999998</v>
+        <v>-8558.620001000001</v>
       </c>
     </row>
     <row r="13">
@@ -10811,10 +11618,10 @@
         <v>12629.390004</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>4952.160010000001</v>
+        <v>4952.16001</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>-7677.229993999998</v>
+        <v>-7677.229994000001</v>
       </c>
     </row>
     <row r="14">
@@ -10856,7 +11663,7 @@
         <v>10528.90002</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>-6146.779965999998</v>
+        <v>-6146.779966</v>
       </c>
     </row>
     <row r="15">
@@ -10895,10 +11702,10 @@
         <v>12714.230007</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>7402.850004999999</v>
+        <v>7402.850005</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>-5311.380002000003</v>
+        <v>-5311.380002</v>
       </c>
     </row>
     <row r="16">
@@ -10976,7 +11783,7 @@
         <v>1.587301587301587</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>5602.800003</v>
+        <v>5602.800003000001</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>1245.960001</v>
@@ -11060,13 +11867,13 @@
         <v>3.472222222222222</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>7115.929990000001</v>
+        <v>7115.92999</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>3963.600001</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>-3152.329989</v>
+        <v>-3152.329988999999</v>
       </c>
     </row>
     <row r="20">
@@ -11264,7 +12071,7 @@
         <v>3.764115432873274</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>26663.18999299999</v>
+        <v>26663.189993</v>
       </c>
       <c r="K24" s="5" t="n">
         <v>35959.800021</v>
@@ -11306,13 +12113,13 @@
         <v>0.5343022013250694</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>44231.229999</v>
+        <v>44231.22999899999</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>56932.93002</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>12701.700021</v>
+        <v>12701.70002100001</v>
       </c>
     </row>
     <row r="26">
@@ -11351,10 +12158,10 @@
         <v>31839.919989</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>49597.55998000001</v>
+        <v>49597.55998</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>17757.63999100001</v>
+        <v>17757.639991</v>
       </c>
     </row>
     <row r="29">
@@ -11408,16 +12215,16 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.640110978993262</v>
+        <v>0.6402378592666006</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.67665719384046</v>
+        <v>0.655596643436211</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>3.6546214847198</v>
+        <v>1.535878416961045</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0.05709356040834712</v>
+        <v>0.02398918456213139</v>
       </c>
     </row>
     <row r="32">
@@ -11435,13 +12242,13 @@
         <v>0.09044670499778859</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>0.1024564145138448</v>
+        <v>0.08748237335936652</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>1.20097095160562</v>
+        <v>-0.2964331638422066</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>0.1327821673144405</v>
+        <v>-0.03277434637883758</v>
       </c>
     </row>
     <row r="33">
@@ -11459,13 +12266,13 @@
         <v>0.7799511002444988</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>0.8317445185891325</v>
+        <v>0.7823930564166151</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>5.179341834463369</v>
+        <v>0.2441956172116289</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0.06640598151396615</v>
+        <v>0.003130909324124076</v>
       </c>
     </row>
     <row r="34">
@@ -11483,13 +12290,13 @@
         <v>0.6858934169278997</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0.5249283667621777</v>
+        <v>0.7258320126782885</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>-16.09650501657221</v>
+        <v>3.993859575038872</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>-0.2346793921520354</v>
+        <v>0.05822857424302552</v>
       </c>
     </row>
     <row r="35">
@@ -11531,13 +12338,13 @@
         <v>0.6156739811912225</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>0.4796561604584527</v>
+        <v>0.6632329635499208</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>-13.60178207327698</v>
+        <v>4.755898235869827</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>-0.2209250754264438</v>
+        <v>0.07724702328118505</v>
       </c>
     </row>
     <row r="37">
@@ -11555,13 +12362,13 @@
         <v>0.04343210968597966</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>0.04087512819260634</v>
+        <v>0.04539537910836317</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>-0.2556981493373321</v>
+        <v>0.1963269422383507</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>-0.05887306676697635</v>
+        <v>0.04520317885956326</v>
       </c>
     </row>
     <row r="38">
@@ -11956,19 +12763,19 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>29882</v>
+        <v>29957</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>0.01184659661334583</v>
+        <v>0.01185031879026605</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>402.78116733787</v>
+        <v>424.1036109772248</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>142584.533237606</v>
+        <v>150556.7818969148</v>
       </c>
     </row>
     <row r="57">
@@ -11983,19 +12790,19 @@
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>7120</v>
+        <v>6886</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.03019662921348315</v>
+        <v>0.03194888178913738</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>383.1614776291792</v>
+        <v>394.8387869800015</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>82379.71769027352</v>
+        <v>86864.53313560033</v>
       </c>
     </row>
     <row r="58">
@@ -12010,19 +12817,19 @@
         </is>
       </c>
       <c r="C58" s="3" t="n">
-        <v>22690</v>
+        <v>22999</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>0.006081974438078449</v>
+        <v>0.005826340275664159</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>434.9740552175549</v>
+        <v>473.8821478191897</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>60026.41962002258</v>
+        <v>63500.20780777142</v>
       </c>
     </row>
     <row r="59">
@@ -12046,10 +12853,10 @@
         <v>0.01388888888888889</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>178.3959273098884</v>
+        <v>192.040953543025</v>
       </c>
       <c r="G59" s="5" t="n">
-        <v>178.3959273098884</v>
+        <v>192.040953543025</v>
       </c>
     </row>
     <row r="60">
@@ -12170,16 +12977,16 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>35799</v>
+        <v>35791</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>396</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>0.01106176150171793</v>
+        <v>0.01106423402531363</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>338.2361110757576</v>
+        <v>338.2361110757577</v>
       </c>
       <c r="G64" s="5" t="n">
         <v>133941.499986</v>
@@ -12197,19 +13004,19 @@
         </is>
       </c>
       <c r="C65" s="3" t="n">
-        <v>7394</v>
+        <v>7386</v>
       </c>
       <c r="D65" s="3" t="n">
         <v>222</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.03002434406275358</v>
+        <v>0.03005686433793664</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>359.4633332252253</v>
+        <v>359.4633332252254</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>79800.85997600001</v>
+        <v>79800.85997600004</v>
       </c>
     </row>
     <row r="66">
@@ -19614,13 +20421,13 @@
         <v>0.008280565026790063</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>887331.6599719999</v>
+        <v>887331.6599720001</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>636151.100001</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-251180.5599709999</v>
+        <v>-251180.5599710001</v>
       </c>
     </row>
     <row r="4">
@@ -19704,7 +20511,7 @@
         <v>8080.720001</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-8558.620000999998</v>
+        <v>-8558.620001000001</v>
       </c>
     </row>
     <row r="7">
@@ -19810,7 +20617,7 @@
         <v>0.02564102564102564</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>9371.580008999999</v>
+        <v>9371.580009000001</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>3676.779999</v>
@@ -19844,7 +20651,7 @@
         <v>11529.589994</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-5145.430019000003</v>
+        <v>-5145.430019</v>
       </c>
     </row>
     <row r="12">
@@ -19984,7 +20791,7 @@
         <v>12039.320007</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-1956.909962999997</v>
+        <v>-1956.909963000001</v>
       </c>
     </row>
     <row r="17">
@@ -20022,25 +20829,25 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>84537</v>
+        <v>84525</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>84217</v>
+        <v>82221</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.01807492577214711</v>
+        <v>0.01807749186631174</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.01765676763598798</v>
+        <v>0.01808540397222121</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>520907.4199640001</v>
+        <v>520907.419964</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>528516.0501550001</v>
+        <v>528516.0501549999</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>7608.630190999966</v>
+        <v>7608.630190999937</v>
       </c>
     </row>
     <row r="19">
@@ -20062,10 +20869,10 @@
         <v>0.0110938540048813</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>29088.47998599999</v>
+        <v>29088.479986</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>39788.29002499999</v>
+        <v>39788.290025</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>10699.810039</v>
@@ -20106,25 +20913,25 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>15824</v>
+        <v>15823</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>17457</v>
+        <v>17437</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.009036905965621841</v>
+        <v>0.009037477090311571</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.01042561723091024</v>
+        <v>0.01043757527097551</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>45234.049987</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>61329.45001100001</v>
+        <v>61329.450011</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>16095.40002400001</v>
+        <v>16095.400024</v>
       </c>
     </row>
     <row r="22">
@@ -20233,13 +21040,13 @@
         <v>0.005970758750409909</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>464426.4899459999</v>
+        <v>464426.489946</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>316076.920068</v>
+        <v>316076.9200679999</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>-148349.5698779999</v>
+        <v>-148349.5698780001</v>
       </c>
     </row>
     <row r="28">
@@ -20371,7 +21178,7 @@
         <v>8080.720001</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>-8558.620000999998</v>
+        <v>-8558.620001000001</v>
       </c>
     </row>
     <row r="32">
@@ -20470,7 +21277,7 @@
         <v>10069.72</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>-5270.880008000003</v>
+        <v>-5270.880008</v>
       </c>
     </row>
     <row r="35">
@@ -20503,7 +21310,7 @@
         <v>17656.220022</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>-5257.039969999999</v>
+        <v>-5257.039970000001</v>
       </c>
     </row>
     <row r="36">
@@ -20596,7 +21403,7 @@
         <v>0.01587301587301587</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>5602.800003</v>
+        <v>5602.800003000001</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>1245.960001</v>
@@ -20922,7 +21729,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>-200378.9800009999</v>
+        <v>-200378.9800010001</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
Refresh workbook with clean Oscar web extraction
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012iFLn21AiUGfBb2WhkxcsV
</commit_message>
<xml_diff>
--- a/analise/Respostas_por_bandeira_set26.xlsx
+++ b/analise/Respostas_por_bandeira_set26.xlsx
@@ -709,10 +709,10 @@
         <v>202605</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>318584</v>
+        <v>318116</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.009501418778093062</v>
+        <v>0.009515396899244301</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>350.6384514182847</v>
@@ -731,13 +731,13 @@
         <v>202606</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>302886</v>
+        <v>302393</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.01064426880080294</v>
+        <v>0.01066162245819182</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>367.7144788566365</v>
+        <v>367.7144788566366</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>1185511.479833796</v>
@@ -753,16 +753,16 @@
         <v>202607</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>344514</v>
+        <v>343842</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.01269904851471929</v>
+        <v>0.01272386735768173</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>401.0144010982897</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1754438.004805017</v>
+        <v>1754438.004805018</v>
       </c>
     </row>
     <row r="6">
@@ -775,10 +775,10 @@
         <v>202608</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>281568</v>
+        <v>280903</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.01107015001704739</v>
+        <v>0.01109635710547769</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>337.6660344742969</v>
@@ -797,10 +797,10 @@
         <v>202609</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>245193</v>
+        <v>243782</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.009506796686691708</v>
+        <v>0.00956182162751967</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>357.483778684379</v>
@@ -819,10 +819,10 @@
         <v>202610</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>29066</v>
+        <v>27666</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.01238560517443061</v>
+        <v>0.01301236174365647</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>372.9152228734548</v>
@@ -1698,10 +1698,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>265721</v>
+        <v>264958</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>188929</v>
+        <v>188152</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>3171</v>
@@ -1710,7 +1710,7 @@
         <v>1074193.889856</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.01193356942055765</v>
+        <v>0.01196793454056869</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>338.7555628684958</v>
@@ -1733,10 +1733,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>58118</v>
+        <v>57355</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>36172</v>
+        <v>35395</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>1567</v>
@@ -1745,7 +1745,7 @@
         <v>554561.2799580001</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.02696238686809594</v>
+        <v>0.02732107052567344</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>353.8999872099554</v>
@@ -1777,13 +1777,13 @@
         <v>1598</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>518071.3098939999</v>
+        <v>518071.309894</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>0.007722045037208853</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>324.1998184568209</v>
+        <v>324.199818456821</v>
       </c>
     </row>
     <row r="6">
@@ -1838,10 +1838,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>247187</v>
+        <v>246120</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>176550</v>
+        <v>175355</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>2521</v>
@@ -1850,7 +1850,7 @@
         <v>887772.7301079999</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0.01019875640709261</v>
+        <v>0.01024297090849992</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>352.1510234462514</v>
@@ -1873,19 +1873,19 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>48055</v>
+        <v>46988</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>28647</v>
+        <v>27452</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1384</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>503337.839989</v>
+        <v>503337.8399889999</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>0.02880033295182603</v>
+        <v>0.02945432876479101</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>363.6834103966763</v>
@@ -1917,13 +1917,13 @@
         <v>1135</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>383624.9101209999</v>
+        <v>383624.910121</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>0.005725989940419435</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>337.99551552511</v>
+        <v>337.9955155251101</v>
       </c>
     </row>
     <row r="10">
@@ -1978,10 +1978,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>29957</v>
+        <v>28647</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>25483</v>
+        <v>24229</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>355</v>
@@ -1990,7 +1990,7 @@
         <v>150556.7818969148</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0.01185031879026605</v>
+        <v>0.01239222257129891</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>424.1036109772248</v>
@@ -2013,10 +2013,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>6886</v>
+        <v>5576</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5410</v>
+        <v>4156</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>220</v>
@@ -2025,7 +2025,7 @@
         <v>86864.53313560033</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0.03194888178913738</v>
+        <v>0.03945480631276901</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>394.8387869800015</v>
@@ -2118,10 +2118,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46497</v>
+        <v>46354</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>38281</v>
+        <v>38124</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>400</v>
@@ -2130,7 +2130,7 @@
         <v>140057.860009</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.008602705550895757</v>
+        <v>0.008629244509643181</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>350.1446500225</v>
@@ -2153,10 +2153,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>6056</v>
+        <v>5913</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>4409</v>
+        <v>4252</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>205</v>
@@ -2165,7 +2165,7 @@
         <v>73974.219996</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.03385072655217965</v>
+        <v>0.03466937256891595</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>360.8498536390244</v>
@@ -2256,10 +2256,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>35791</v>
+        <v>35357</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>29387</v>
+        <v>28989</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>396</v>
@@ -2268,10 +2268,10 @@
         <v>133941.499986</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.01106423402531363</v>
+        <v>0.01120004525270809</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>338.2361110757577</v>
+        <v>338.2361110757576</v>
       </c>
     </row>
     <row r="20">
@@ -2291,22 +2291,22 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>7386</v>
+        <v>6952</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>5022</v>
+        <v>4624</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>222</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>79800.85997600004</v>
+        <v>79800.85997600001</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.03005686433793664</v>
+        <v>0.03193325661680092</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>359.4633332252254</v>
+        <v>359.4633332252253</v>
       </c>
     </row>
     <row r="21">
@@ -5086,25 +5086,25 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.6402378592666006</v>
+        <v>0.6472138554216867</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>0.655596643436211</v>
+        <v>0.6753208218974853</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1.535878416961045</v>
+        <v>2.810696647579858</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>0.02398918456213139</v>
+        <v>0.04342763406615524</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>0.4357875116495806</v>
+        <v>0.5352798053527981</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>0.6356011183597391</v>
+        <v>0.6455665619714906</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>0.5868592351505288</v>
+        <v>0.6334070796460177</v>
       </c>
     </row>
     <row r="4">
@@ -5124,25 +5124,25 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.09044670499778859</v>
+        <v>0.09151116480959413</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.08748237335936652</v>
+        <v>0.08858743409490334</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>-0.2964331638422066</v>
+        <v>-0.2923730714690792</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>-0.03277434637883758</v>
+        <v>-0.03194944268029098</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.08554319931565441</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>0.08357771260997067</v>
+        <v>0.08532934131736528</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>0.1081455805892548</v>
+        <v>0.108976597974153</v>
       </c>
     </row>
     <row r="5">
@@ -5281,25 +5281,25 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0.04343210968597966</v>
+        <v>0.04394325860294446</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.04539537910836317</v>
+        <v>0.04596880492091388</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.1963269422383507</v>
+        <v>0.2025546317969418</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.04520317885956326</v>
+        <v>0.04609458611778261</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.07570573139435414</v>
+        <v>0.08045454545454546</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.05865102639296188</v>
+        <v>0.05988023952095808</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0.058578856152513</v>
+        <v>0.05902899056933287</v>
       </c>
     </row>
     <row r="9">
@@ -5319,25 +5319,25 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.07054400707651481</v>
+        <v>0.07137423367789859</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.06844560147521424</v>
+        <v>0.06931019332161688</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>-0.2098405601300576</v>
+        <v>-0.2064040356281716</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>-0.02974605056138313</v>
+        <v>-0.02891856416415517</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>0.05603079555175364</v>
+        <v>0.05954545454545455</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.06634897360703812</v>
+        <v>0.06773952095808383</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>0.08700173310225304</v>
+        <v>0.08767027593433462</v>
       </c>
     </row>
     <row r="10">
@@ -7837,16 +7837,16 @@
         </is>
       </c>
       <c r="D77" s="6" t="n">
-        <v>0.6449035552193646</v>
+        <v>0.6488056295776221</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>0.6531370691539751</v>
+        <v>0.6629815745393635</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>0.823351393461047</v>
+        <v>1.417594496174135</v>
       </c>
       <c r="G77" s="6" t="n">
-        <v>0.01276704689867914</v>
+        <v>0.02184929401887281</v>
       </c>
     </row>
     <row r="78">
@@ -7866,16 +7866,16 @@
         </is>
       </c>
       <c r="D78" s="6" t="n">
-        <v>0.07919751728856633</v>
+        <v>0.07970978848991637</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>0.07742943210978467</v>
+        <v>0.07792936949076414</v>
       </c>
       <c r="F78" s="7" t="n">
-        <v>-0.1768085178781659</v>
+        <v>-0.1780418999152239</v>
       </c>
       <c r="G78" s="6" t="n">
-        <v>-0.02232500764309842</v>
+        <v>-0.02233626550618018</v>
       </c>
     </row>
     <row r="79">
@@ -7982,16 +7982,16 @@
         </is>
       </c>
       <c r="D82" s="6" t="n">
-        <v>0.03157148791633067</v>
+        <v>0.03177570093457944</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>0.03045855182416602</v>
+        <v>0.03065521307057436</v>
       </c>
       <c r="F82" s="7" t="n">
-        <v>-0.1112936092164649</v>
+        <v>-0.1120487864005076</v>
       </c>
       <c r="G82" s="6" t="n">
-        <v>-0.03525130317310676</v>
+        <v>-0.03526241219074799</v>
       </c>
     </row>
     <row r="83">
@@ -8301,10 +8301,10 @@
         <v>0.004721504979712283</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-6664.843679511983</v>
+        <v>-6664.843679511989</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>-6433.363660511985</v>
+        <v>-6433.363660511986</v>
       </c>
     </row>
     <row r="4">
@@ -8343,10 +8343,10 @@
         <v>0.03122130394857667</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-6242.8731032826</v>
+        <v>-6242.873103282596</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>-5161.403098282593</v>
+        <v>-5161.40309828259</v>
       </c>
     </row>
     <row r="5">
@@ -8679,10 +8679,10 @@
         <v>0.03630363036303631</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>6606.576998513947</v>
+        <v>6606.576998513949</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>4489.347000513947</v>
+        <v>4489.347000513949</v>
       </c>
     </row>
     <row r="13">
@@ -8697,13 +8697,13 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2414</v>
+        <v>1160</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>796</v>
+        <v>725</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1257</v>
+        <v>874</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>107</v>
@@ -8715,10 +8715,10 @@
         <v>90</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>0.04432477216238608</v>
+        <v>0.09224137931034483</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.07159904534606205</v>
+        <v>0.102974828375286</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>8800.547034558862</v>
@@ -8766,7 +8766,7 @@
         <v>11842.27878525751</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>6494.538780257517</v>
+        <v>6494.538780257513</v>
       </c>
     </row>
     <row r="15"/>
@@ -10638,19 +10638,19 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>265721</v>
+        <v>264958</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>247187</v>
+        <v>246120</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-0.06974985040700588</v>
+        <v>-0.07109806082473447</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.01193356942055765</v>
+        <v>0.01196793454056869</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.01019875640709261</v>
+        <v>0.01024297090849992</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>338.7555628684958</v>
@@ -10680,16 +10680,16 @@
         <v>-207184</v>
       </c>
       <c r="P3" s="5" t="n">
-        <v>-49759.8222797596</v>
+        <v>-50721.64098460888</v>
       </c>
       <c r="Q3" s="5" t="n">
-        <v>-96475.62395171315</v>
+        <v>-95513.80524686385</v>
       </c>
       <c r="R3" s="5" t="n">
-        <v>22427.62875571827</v>
+        <v>22427.62875571817</v>
       </c>
       <c r="S3" s="5" t="n">
-        <v>-83376.1825242456</v>
+        <v>-83376.18252424549</v>
       </c>
     </row>
     <row r="4">
@@ -11078,13 +11078,13 @@
         <v>465538</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>501269</v>
+        <v>500202</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>0.013</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.009136537658294069</v>
+        <v>0.009156027155899835</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>300</v>
@@ -11099,10 +11099,10 @@
         <v>1237130.99</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>139350.9</v>
+        <v>135189.6</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-580990.1713693771</v>
+        <v>-576828.8713693771</v>
       </c>
       <c r="L3" s="5" t="n">
         <v>244257.2450402343</v>
@@ -11181,7 +11181,7 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11265,19 +11265,19 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>58118</v>
+        <v>57355</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>48055</v>
+        <v>46988</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>-0.1731477339206442</v>
+        <v>-0.1807514602039927</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.02696238686809594</v>
+        <v>0.02732107052567344</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.02880033295182603</v>
+        <v>0.02945432876479101</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>353.8999872099554</v>
@@ -11289,16 +11289,16 @@
         <v>554561.2799580001</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>503337.8399890001</v>
+        <v>503337.8399889999</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-96021.02894485969</v>
+        <v>-100237.7611250037</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>31257.33128543783</v>
+        <v>35474.06346558184</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>13540.25769042178</v>
+        <v>13540.2576904217</v>
       </c>
     </row>
     <row r="4">
@@ -11323,16 +11323,16 @@
         <v>0.005725989940419435</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>324.1998184568209</v>
+        <v>324.199818456821</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>337.99551552511</v>
+        <v>337.9955155251101</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>518071.3098939998</v>
+        <v>518071.3098940001</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>383624.9101209998</v>
+        <v>383624.910121</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>-21832.89791043575</v>
@@ -11341,7 +11341,7 @@
         <v>-128271.6180350724</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>15658.11617250811</v>
+        <v>15658.11617250805</v>
       </c>
     </row>
     <row r="5">
@@ -11489,13 +11489,13 @@
         <v>0.4623795997693441</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>264189.8699630001</v>
+        <v>264189.869963</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>135106.590022</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>-129083.2799410001</v>
+        <v>-129083.279941</v>
       </c>
     </row>
     <row r="11">
@@ -11537,7 +11537,7 @@
         <v>148207.179955</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>-70431.75005499998</v>
+        <v>-70431.75005500001</v>
       </c>
     </row>
     <row r="12">
@@ -11618,10 +11618,10 @@
         <v>12629.390004</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>4952.16001</v>
+        <v>4952.160010000001</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>-7677.229994000001</v>
+        <v>-7677.229993999998</v>
       </c>
     </row>
     <row r="14">
@@ -11663,7 +11663,7 @@
         <v>10528.90002</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>-6146.779966</v>
+        <v>-6146.779966000004</v>
       </c>
     </row>
     <row r="15">
@@ -11702,10 +11702,10 @@
         <v>12714.230007</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>7402.850005</v>
+        <v>7402.850004999999</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>-5311.380002</v>
+        <v>-5311.380002000003</v>
       </c>
     </row>
     <row r="16">
@@ -11741,13 +11741,13 @@
         <v>1.520912547528517</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>5736.079991000001</v>
+        <v>5736.079991</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>1063.779998</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>-4672.299993000001</v>
+        <v>-4672.299993</v>
       </c>
     </row>
     <row r="17">
@@ -11783,7 +11783,7 @@
         <v>1.587301587301587</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>5602.800003000001</v>
+        <v>5602.800003</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>1245.960001</v>
@@ -11825,13 +11825,13 @@
         <v>0</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>3461.879999</v>
+        <v>3461.879999000001</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>-3461.879999</v>
+        <v>-3461.879999000001</v>
       </c>
     </row>
     <row r="19">
@@ -11867,13 +11867,13 @@
         <v>3.472222222222222</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>7115.92999</v>
+        <v>7115.929990000001</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>3963.600001</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>-3152.329988999999</v>
+        <v>-3152.329989</v>
       </c>
     </row>
     <row r="20">
@@ -11915,7 +11915,7 @@
         <v>614.980001</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>-2832.930006000001</v>
+        <v>-2832.930006</v>
       </c>
     </row>
     <row r="21">
@@ -12035,7 +12035,7 @@
         <v>132934.42002</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>5556.870077</v>
+        <v>5556.87007699997</v>
       </c>
     </row>
     <row r="24">
@@ -12113,13 +12113,13 @@
         <v>0.5343022013250694</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>44231.22999899999</v>
+        <v>44231.22999900001</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>56932.93002</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>12701.70002100001</v>
+        <v>12701.70002099999</v>
       </c>
     </row>
     <row r="26">
@@ -12215,16 +12215,16 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.6402378592666006</v>
+        <v>0.6472138554216867</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.655596643436211</v>
+        <v>0.6753208218974853</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>1.535878416961045</v>
+        <v>2.810696647579858</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0.02398918456213139</v>
+        <v>0.04342763406615524</v>
       </c>
     </row>
     <row r="32">
@@ -12239,16 +12239,16 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0.09044670499778859</v>
+        <v>0.09151116480959413</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>0.08748237335936652</v>
+        <v>0.08858743409490334</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>-0.2964331638422066</v>
+        <v>-0.2923730714690792</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>-0.03277434637883758</v>
+        <v>-0.03194944268029098</v>
       </c>
     </row>
     <row r="33">
@@ -12359,16 +12359,16 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>0.04343210968597966</v>
+        <v>0.04394325860294446</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>0.04539537910836317</v>
+        <v>0.04596880492091388</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.1963269422383507</v>
+        <v>0.2025546317969418</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0.04520317885956326</v>
+        <v>0.04609458611778261</v>
       </c>
     </row>
     <row r="38">
@@ -12763,13 +12763,13 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>29957</v>
+        <v>28647</v>
       </c>
       <c r="D56" s="3" t="n">
         <v>355</v>
       </c>
       <c r="E56" s="4" t="n">
-        <v>0.01185031879026605</v>
+        <v>0.01239222257129891</v>
       </c>
       <c r="F56" s="5" t="n">
         <v>424.1036109772248</v>
@@ -12790,13 +12790,13 @@
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>6886</v>
+        <v>5576</v>
       </c>
       <c r="D57" s="3" t="n">
         <v>220</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.03194888178913738</v>
+        <v>0.03945480631276901</v>
       </c>
       <c r="F57" s="5" t="n">
         <v>394.8387869800015</v>
@@ -12871,13 +12871,13 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>46497</v>
+        <v>46354</v>
       </c>
       <c r="D60" s="3" t="n">
         <v>400</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>0.008602705550895757</v>
+        <v>0.008629244509643181</v>
       </c>
       <c r="F60" s="5" t="n">
         <v>350.1446500225</v>
@@ -12898,13 +12898,13 @@
         </is>
       </c>
       <c r="C61" s="3" t="n">
-        <v>6056</v>
+        <v>5913</v>
       </c>
       <c r="D61" s="3" t="n">
         <v>205</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>0.03385072655217965</v>
+        <v>0.03466937256891595</v>
       </c>
       <c r="F61" s="5" t="n">
         <v>360.8498536390244</v>
@@ -12977,16 +12977,16 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>35791</v>
+        <v>35357</v>
       </c>
       <c r="D64" s="3" t="n">
         <v>396</v>
       </c>
       <c r="E64" s="4" t="n">
-        <v>0.01106423402531363</v>
+        <v>0.01120004525270809</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>338.2361110757577</v>
+        <v>338.2361110757576</v>
       </c>
       <c r="G64" s="5" t="n">
         <v>133941.499986</v>
@@ -13004,19 +13004,19 @@
         </is>
       </c>
       <c r="C65" s="3" t="n">
-        <v>7386</v>
+        <v>6952</v>
       </c>
       <c r="D65" s="3" t="n">
         <v>222</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.03005686433793664</v>
+        <v>0.03193325661680092</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>359.4633332252254</v>
+        <v>359.4633332252253</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>79800.85997600004</v>
+        <v>79800.85997600001</v>
       </c>
     </row>
     <row r="66">
@@ -20421,13 +20421,13 @@
         <v>0.008280565026790063</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>887331.6599720001</v>
+        <v>887331.6599719999</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>636151.100001</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-251180.5599710001</v>
+        <v>-251180.559971</v>
       </c>
     </row>
     <row r="4">
@@ -20617,7 +20617,7 @@
         <v>0.02564102564102564</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>9371.580009000001</v>
+        <v>9371.580008999999</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>3676.779999</v>
@@ -20651,7 +20651,7 @@
         <v>11529.589994</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-5145.430019</v>
+        <v>-5145.430019000003</v>
       </c>
     </row>
     <row r="12">
@@ -20679,7 +20679,7 @@
         <v>8244.420017</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-4608.509982</v>
+        <v>-4608.509982000001</v>
       </c>
     </row>
     <row r="13">
@@ -20791,7 +20791,7 @@
         <v>12039.320007</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-1956.909963000001</v>
+        <v>-1956.909962999999</v>
       </c>
     </row>
     <row r="17">
@@ -20829,16 +20829,16 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>84525</v>
+        <v>84152</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>82221</v>
+        <v>81358</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.01807749186631174</v>
+        <v>0.01815761954558418</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.01808540397222121</v>
+        <v>0.01827724378672042</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>520907.419964</v>
@@ -20913,19 +20913,19 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>15823</v>
+        <v>15480</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>17437</v>
+        <v>17064</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0.009037477090311571</v>
+        <v>0.009237726098191214</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.01043757527097551</v>
+        <v>0.0106657290201594</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>45234.049987</v>
+        <v>45234.04998700001</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>61329.450011</v>
@@ -20959,7 +20959,7 @@
         <v>159039.490009</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>30955.63998900001</v>
+        <v>30955.63998899999</v>
       </c>
     </row>
     <row r="25">
@@ -21043,10 +21043,10 @@
         <v>464426.489946</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>316076.9200679999</v>
+        <v>316076.920068</v>
       </c>
       <c r="I27" s="5" t="n">
-        <v>-148349.5698780001</v>
+        <v>-148349.569878</v>
       </c>
     </row>
     <row r="28">
@@ -21079,7 +21079,7 @@
         <v>212867.689981</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-73051.39000899998</v>
+        <v>-73051.39000900001</v>
       </c>
     </row>
     <row r="29">
@@ -21277,7 +21277,7 @@
         <v>10069.72</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>-5270.880008</v>
+        <v>-5270.880008000003</v>
       </c>
     </row>
     <row r="35">
@@ -21310,7 +21310,7 @@
         <v>17656.220022</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>-5257.039970000001</v>
+        <v>-5257.039970000004</v>
       </c>
     </row>
     <row r="36">
@@ -21370,13 +21370,13 @@
         <v>0.01520912547528517</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>5736.079991000001</v>
+        <v>5736.079991</v>
       </c>
       <c r="H37" s="5" t="n">
         <v>1063.779998</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>-4672.299993000001</v>
+        <v>-4672.299993</v>
       </c>
     </row>
     <row r="38">
@@ -21403,7 +21403,7 @@
         <v>0.01587301587301587</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>5602.800003000001</v>
+        <v>5602.800003</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>1245.960001</v>
@@ -21729,7 +21729,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>-200378.9800010001</v>
+        <v>-200378.980001</v>
       </c>
     </row>
     <row r="58">

</xml_diff>